<commit_message>
Replace placeholders in NGFW project plan with defaults
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Nd9zRhMDNGo9krQcisnhME
</commit_message>
<xml_diff>
--- a/deliverables/NGFW_Maturity_Project_Plan.xlsx
+++ b/deliverables/NGFW_Maturity_Project_Plan.xlsx
@@ -3887,7 +3887,7 @@
       </c>
       <c r="H4" s="48" t="inlineStr">
         <is>
-          <t>[Network Security Lead]</t>
+          <t>Network Security Lead</t>
         </is>
       </c>
       <c r="I4" s="11">
@@ -3931,7 +3931,7 @@
       </c>
       <c r="H5" s="48" t="inlineStr">
         <is>
-          <t>[CISO / Sponsor]</t>
+          <t>CISO</t>
         </is>
       </c>
       <c r="I5" s="11">
@@ -3975,7 +3975,7 @@
       </c>
       <c r="H6" s="48" t="inlineStr">
         <is>
-          <t>[CISO / Sponsor]</t>
+          <t>CISO</t>
         </is>
       </c>
       <c r="I6" s="11">
@@ -4019,7 +4019,7 @@
       </c>
       <c r="H7" s="48" t="inlineStr">
         <is>
-          <t>[Executive Sponsor]</t>
+          <t>Executive Sponsor</t>
         </is>
       </c>
       <c r="I7" s="11">
@@ -5062,7 +5062,7 @@
       </c>
       <c r="B3" s="56" t="inlineStr">
         <is>
-          <t>[Client Name]</t>
+          <t>Customer</t>
         </is>
       </c>
     </row>
@@ -5117,7 +5117,7 @@
       </c>
       <c r="B8" s="56" t="inlineStr">
         <is>
-          <t>[Consulting Lead]</t>
+          <t>Engagement Lead</t>
         </is>
       </c>
     </row>
@@ -5129,7 +5129,7 @@
       </c>
       <c r="B9" s="56" t="inlineStr">
         <is>
-          <t>[Client Sponsor]</t>
+          <t>CISO</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Compress assessment deliverables into first 4 weeks; add remediation execution phases
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Nd9zRhMDNGo9krQcisnhME
</commit_message>
<xml_diff>
--- a/deliverables/NGFW_Maturity_Project_Plan.xlsx
+++ b/deliverables/NGFW_Maturity_Project_Plan.xlsx
@@ -804,7 +804,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F22"/>
+  <dimension ref="A1:F24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -890,7 +890,7 @@
         </is>
       </c>
       <c r="B9" s="6">
-        <f>'Project Plan'!G46</f>
+        <f>'Project Plan'!G51</f>
         <v/>
       </c>
     </row>
@@ -901,7 +901,7 @@
         </is>
       </c>
       <c r="B10" s="5">
-        <f>COUNTIF('Project Plan'!H5:H44,"Late")+COUNTIF('Project Plan'!H5:H44,"Late Start")</f>
+        <f>COUNTIF('Project Plan'!H5:H49,"Late")+COUNTIF('Project Plan'!H5:H49,"Late Start")</f>
         <v/>
       </c>
     </row>
@@ -1009,117 +1009,169 @@
     </row>
     <row r="17">
       <c r="A17" s="9">
-        <f>'Project Plan'!B19</f>
+        <f>'Project Plan'!B17</f>
         <v/>
       </c>
       <c r="B17" s="10">
-        <f>'Project Plan'!D19</f>
+        <f>'Project Plan'!D17</f>
         <v/>
       </c>
       <c r="C17" s="10">
-        <f>'Project Plan'!E19</f>
+        <f>'Project Plan'!E17</f>
         <v/>
       </c>
       <c r="D17" s="11">
-        <f>'Project Plan'!F19</f>
+        <f>'Project Plan'!F17</f>
         <v/>
       </c>
       <c r="E17" s="12">
-        <f>'Project Plan'!G19</f>
+        <f>'Project Plan'!G17</f>
         <v/>
       </c>
       <c r="F17" s="11">
-        <f>'Project Plan'!H19</f>
+        <f>'Project Plan'!H17</f>
         <v/>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="9">
-        <f>'Project Plan'!B27</f>
+        <f>'Project Plan'!B23</f>
         <v/>
       </c>
       <c r="B18" s="10">
-        <f>'Project Plan'!D27</f>
+        <f>'Project Plan'!D23</f>
         <v/>
       </c>
       <c r="C18" s="10">
-        <f>'Project Plan'!E27</f>
+        <f>'Project Plan'!E23</f>
         <v/>
       </c>
       <c r="D18" s="11">
-        <f>'Project Plan'!F27</f>
+        <f>'Project Plan'!F23</f>
         <v/>
       </c>
       <c r="E18" s="12">
-        <f>'Project Plan'!G27</f>
+        <f>'Project Plan'!G23</f>
         <v/>
       </c>
       <c r="F18" s="11">
-        <f>'Project Plan'!H27</f>
+        <f>'Project Plan'!H23</f>
         <v/>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="9">
-        <f>'Project Plan'!B34</f>
+        <f>'Project Plan'!B27</f>
         <v/>
       </c>
       <c r="B19" s="10">
-        <f>'Project Plan'!D34</f>
+        <f>'Project Plan'!D27</f>
         <v/>
       </c>
       <c r="C19" s="10">
-        <f>'Project Plan'!E34</f>
+        <f>'Project Plan'!E27</f>
         <v/>
       </c>
       <c r="D19" s="11">
-        <f>'Project Plan'!F34</f>
+        <f>'Project Plan'!F27</f>
         <v/>
       </c>
       <c r="E19" s="12">
-        <f>'Project Plan'!G34</f>
+        <f>'Project Plan'!G27</f>
         <v/>
       </c>
       <c r="F19" s="11">
-        <f>'Project Plan'!H34</f>
+        <f>'Project Plan'!H27</f>
         <v/>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="9">
-        <f>'Project Plan'!B40</f>
+        <f>'Project Plan'!B31</f>
         <v/>
       </c>
       <c r="B20" s="10">
-        <f>'Project Plan'!D40</f>
+        <f>'Project Plan'!D31</f>
         <v/>
       </c>
       <c r="C20" s="10">
-        <f>'Project Plan'!E40</f>
+        <f>'Project Plan'!E31</f>
         <v/>
       </c>
       <c r="D20" s="11">
-        <f>'Project Plan'!F40</f>
+        <f>'Project Plan'!F31</f>
         <v/>
       </c>
       <c r="E20" s="12">
-        <f>'Project Plan'!G40</f>
+        <f>'Project Plan'!G31</f>
         <v/>
       </c>
       <c r="F20" s="11">
-        <f>'Project Plan'!H40</f>
+        <f>'Project Plan'!H31</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="9">
+        <f>'Project Plan'!B35</f>
+        <v/>
+      </c>
+      <c r="B21" s="10">
+        <f>'Project Plan'!D35</f>
+        <v/>
+      </c>
+      <c r="C21" s="10">
+        <f>'Project Plan'!E35</f>
+        <v/>
+      </c>
+      <c r="D21" s="11">
+        <f>'Project Plan'!F35</f>
+        <v/>
+      </c>
+      <c r="E21" s="12">
+        <f>'Project Plan'!G35</f>
+        <v/>
+      </c>
+      <c r="F21" s="11">
+        <f>'Project Plan'!H35</f>
         <v/>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="13" t="inlineStr">
-        <is>
-          <t>Methodology: Discovery → Pain Points / Gaps → Future-State Vision → Remediation Plan &amp; Roadmap → Readout</t>
+      <c r="A22" s="9">
+        <f>'Project Plan'!B44</f>
+        <v/>
+      </c>
+      <c r="B22" s="10">
+        <f>'Project Plan'!D44</f>
+        <v/>
+      </c>
+      <c r="C22" s="10">
+        <f>'Project Plan'!E44</f>
+        <v/>
+      </c>
+      <c r="D22" s="11">
+        <f>'Project Plan'!F44</f>
+        <v/>
+      </c>
+      <c r="E22" s="12">
+        <f>'Project Plan'!G44</f>
+        <v/>
+      </c>
+      <c r="F22" s="11">
+        <f>'Project Plan'!H44</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="13" t="inlineStr">
+        <is>
+          <t>Methodology: Weeks 1–4 Discovery → Gaps → Future State → Roadmap &amp; Readout  |  Weeks 5–16 Remediation → Validation &amp; Closeout</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="E15:E20">
+  <conditionalFormatting sqref="E15:E22">
     <cfRule type="dataBar" priority="1">
       <dataBar>
         <cfvo type="num" val="0"/>
@@ -1138,7 +1190,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AA55"/>
+  <dimension ref="A1:AA60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1485,7 +1537,7 @@
         <v>46281</v>
       </c>
       <c r="E8" s="24" t="n">
-        <v>46290</v>
+        <v>46283</v>
       </c>
       <c r="F8" s="21">
         <f>NETWORKDAYS(D8,E8,Inputs!$A$16:$A$21)</f>
@@ -1553,7 +1605,7 @@
         <v/>
       </c>
       <c r="G9" s="25" t="n">
-        <v>0.1</v>
+        <v>0.15</v>
       </c>
       <c r="H9" s="21">
         <f>IF(G9&gt;=1,"Complete",IF(E9&lt;Inputs!$B$7,"Late",IF(G9&gt;0,"In Progress",IF(D9&lt;=Inputs!$B$7,"Late Start","Not Started"))))</f>
@@ -1600,11 +1652,11 @@
       </c>
       <c r="C10" s="17" t="inlineStr"/>
       <c r="D10" s="18">
-        <f>MIN(D11:D18)</f>
+        <f>MIN(D11:D16)</f>
         <v/>
       </c>
       <c r="E10" s="18">
-        <f>MAX(E11:E18)</f>
+        <f>MAX(E11:E16)</f>
         <v/>
       </c>
       <c r="F10" s="17">
@@ -1612,7 +1664,7 @@
         <v/>
       </c>
       <c r="G10" s="19">
-        <f>IFERROR(SUMPRODUCT(F11:F18,G11:G18)/SUM(F11:F18),0)</f>
+        <f>IFERROR(SUMPRODUCT(F11:F16,G11:G16)/SUM(F11:F16),0)</f>
         <v/>
       </c>
       <c r="H10" s="17">
@@ -1656,17 +1708,17 @@
         </is>
       </c>
       <c r="D11" s="24" t="n">
-        <v>46286</v>
+        <v>46281</v>
       </c>
       <c r="E11" s="24" t="n">
-        <v>46297</v>
+        <v>46287</v>
       </c>
       <c r="F11" s="21">
         <f>NETWORKDAYS(D11,E11,Inputs!$A$16:$A$21)</f>
         <v/>
       </c>
       <c r="G11" s="25" t="n">
-        <v>0.6</v>
+        <v>1</v>
       </c>
       <c r="H11" s="21">
         <f>IF(G11&gt;=1,"Complete",IF(E11&lt;Inputs!$B$7,"Late",IF(G11&gt;0,"In Progress",IF(D11&lt;=Inputs!$B$7,"Late Start","Not Started"))))</f>
@@ -1717,17 +1769,17 @@
         </is>
       </c>
       <c r="D12" s="24" t="n">
-        <v>46286</v>
+        <v>46281</v>
       </c>
       <c r="E12" s="24" t="n">
-        <v>46297</v>
+        <v>46287</v>
       </c>
       <c r="F12" s="21">
         <f>NETWORKDAYS(D12,E12,Inputs!$A$16:$A$21)</f>
         <v/>
       </c>
       <c r="G12" s="25" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="H12" s="21">
         <f>IF(G12&gt;=1,"Complete",IF(E12&lt;Inputs!$B$7,"Late",IF(G12&gt;0,"In Progress",IF(D12&lt;=Inputs!$B$7,"Late Start","Not Started"))))</f>
@@ -1778,17 +1830,17 @@
         </is>
       </c>
       <c r="D13" s="24" t="n">
-        <v>46288</v>
+        <v>46281</v>
       </c>
       <c r="E13" s="24" t="n">
-        <v>46301</v>
+        <v>46286</v>
       </c>
       <c r="F13" s="21">
         <f>NETWORKDAYS(D13,E13,Inputs!$A$16:$A$21)</f>
         <v/>
       </c>
       <c r="G13" s="25" t="n">
-        <v>0.4</v>
+        <v>1</v>
       </c>
       <c r="H13" s="21">
         <f>IF(G13&gt;=1,"Complete",IF(E13&lt;Inputs!$B$7,"Late",IF(G13&gt;0,"In Progress",IF(D13&lt;=Inputs!$B$7,"Late Start","Not Started"))))</f>
@@ -1839,17 +1891,17 @@
         </is>
       </c>
       <c r="D14" s="24" t="n">
-        <v>46293</v>
+        <v>46286</v>
       </c>
       <c r="E14" s="24" t="n">
-        <v>46304</v>
+        <v>46289</v>
       </c>
       <c r="F14" s="21">
         <f>NETWORKDAYS(D14,E14,Inputs!$A$16:$A$21)</f>
         <v/>
       </c>
       <c r="G14" s="25" t="n">
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="H14" s="21">
         <f>IF(G14&gt;=1,"Complete",IF(E14&lt;Inputs!$B$7,"Late",IF(G14&gt;0,"In Progress",IF(D14&lt;=Inputs!$B$7,"Late Start","Not Started"))))</f>
@@ -1891,7 +1943,7 @@
       </c>
       <c r="B15" s="22" t="inlineStr">
         <is>
-          <t>Operational process review (change mgmt, rule lifecycle, monitoring)</t>
+          <t>Operational process &amp; tooling review (change mgmt, SIEM, NAC, IdP)</t>
         </is>
       </c>
       <c r="C15" s="23" t="inlineStr">
@@ -1900,17 +1952,17 @@
         </is>
       </c>
       <c r="D15" s="24" t="n">
-        <v>46300</v>
+        <v>46287</v>
       </c>
       <c r="E15" s="24" t="n">
-        <v>46309</v>
+        <v>46290</v>
       </c>
       <c r="F15" s="21">
         <f>NETWORKDAYS(D15,E15,Inputs!$A$16:$A$21)</f>
         <v/>
       </c>
       <c r="G15" s="25" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H15" s="21">
         <f>IF(G15&gt;=1,"Complete",IF(E15&lt;Inputs!$B$7,"Late",IF(G15&gt;0,"In Progress",IF(D15&lt;=Inputs!$B$7,"Late Start","Not Started"))))</f>
@@ -1941,45 +1993,49 @@
       <c r="AA15" s="20" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="21" t="inlineStr">
+      <c r="A16" s="27" t="inlineStr">
         <is>
           <t>1.6</t>
         </is>
       </c>
-      <c r="B16" s="22" t="inlineStr">
-        <is>
-          <t>Tooling &amp; integration review (SIEM, NAC, IdP, orchestration)</t>
-        </is>
-      </c>
-      <c r="C16" s="23" t="inlineStr">
+      <c r="B16" s="28" t="inlineStr">
+        <is>
+          <t>DELIVERABLE: Firewall Estate Architecture (current state)</t>
+        </is>
+      </c>
+      <c r="C16" s="29" t="inlineStr">
         <is>
           <t>Consultant</t>
         </is>
       </c>
-      <c r="D16" s="24" t="n">
-        <v>46300</v>
-      </c>
-      <c r="E16" s="24" t="n">
-        <v>46309</v>
-      </c>
-      <c r="F16" s="21">
+      <c r="D16" s="30" t="n">
+        <v>46289</v>
+      </c>
+      <c r="E16" s="30" t="n">
+        <v>46294</v>
+      </c>
+      <c r="F16" s="27">
         <f>NETWORKDAYS(D16,E16,Inputs!$A$16:$A$21)</f>
         <v/>
       </c>
-      <c r="G16" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="H16" s="21">
+      <c r="G16" s="31" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H16" s="27">
         <f>IF(G16&gt;=1,"Complete",IF(E16&lt;Inputs!$B$7,"Late",IF(G16&gt;0,"In Progress",IF(D16&lt;=Inputs!$B$7,"Late Start","Not Started"))))</f>
         <v/>
       </c>
-      <c r="I16" s="23" t="inlineStr">
-        <is>
-          <t>1.1</t>
-        </is>
-      </c>
-      <c r="J16" s="26" t="inlineStr"/>
-      <c r="K16" s="26" t="inlineStr"/>
+      <c r="I16" s="29" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="J16" s="32" t="inlineStr">
+        <is>
+          <t>D1 – Firewall Estate Architecture</t>
+        </is>
+      </c>
+      <c r="K16" s="32" t="inlineStr"/>
       <c r="L16" s="20" t="n"/>
       <c r="M16" s="20" t="n"/>
       <c r="N16" s="20" t="n"/>
@@ -1998,49 +2054,40 @@
       <c r="AA16" s="20" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="27" t="inlineStr">
-        <is>
-          <t>1.7</t>
-        </is>
-      </c>
-      <c r="B17" s="28" t="inlineStr">
-        <is>
-          <t>DELIVERABLE: Firewall Estate Architecture (current state)</t>
-        </is>
-      </c>
-      <c r="C17" s="29" t="inlineStr">
-        <is>
-          <t>Consultant</t>
-        </is>
-      </c>
-      <c r="D17" s="30" t="n">
-        <v>46304</v>
-      </c>
-      <c r="E17" s="30" t="n">
-        <v>46311</v>
-      </c>
-      <c r="F17" s="27">
+      <c r="A17" s="17" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Phase 2 – Identify Pain Points, Issues &amp; Gaps</t>
+        </is>
+      </c>
+      <c r="C17" s="17" t="inlineStr"/>
+      <c r="D17" s="18">
+        <f>MIN(D18:D22)</f>
+        <v/>
+      </c>
+      <c r="E17" s="18">
+        <f>MAX(E18:E22)</f>
+        <v/>
+      </c>
+      <c r="F17" s="17">
         <f>NETWORKDAYS(D17,E17,Inputs!$A$16:$A$21)</f>
         <v/>
       </c>
-      <c r="G17" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="H17" s="27">
-        <f>IF(G17&gt;=1,"Complete",IF(E17&lt;Inputs!$B$7,"Late",IF(G17&gt;0,"In Progress",IF(D17&lt;=Inputs!$B$7,"Late Start","Not Started"))))</f>
-        <v/>
-      </c>
-      <c r="I17" s="29" t="inlineStr">
-        <is>
-          <t>1.4</t>
-        </is>
-      </c>
-      <c r="J17" s="32" t="inlineStr">
-        <is>
-          <t>D1 – Firewall Estate Architecture</t>
-        </is>
-      </c>
-      <c r="K17" s="32" t="inlineStr"/>
+      <c r="G17" s="19">
+        <f>IFERROR(SUMPRODUCT(F18:F22,G18:G22)/SUM(F18:F22),0)</f>
+        <v/>
+      </c>
+      <c r="H17" s="17">
+        <f>IF(G17&gt;=1,"Complete",IF(G17&gt;0,"In Progress","Not Started"))</f>
+        <v/>
+      </c>
+      <c r="I17" s="17" t="n"/>
+      <c r="J17" s="3" t="n"/>
+      <c r="K17" s="3" t="n"/>
       <c r="L17" s="20" t="n"/>
       <c r="M17" s="20" t="n"/>
       <c r="N17" s="20" t="n"/>
@@ -2059,49 +2106,45 @@
       <c r="AA17" s="20" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="27" t="inlineStr">
-        <is>
-          <t>1.8</t>
-        </is>
-      </c>
-      <c r="B18" s="33" t="inlineStr">
-        <is>
-          <t>Milestone: Discovery complete / D1 review</t>
-        </is>
-      </c>
-      <c r="C18" s="29" t="inlineStr">
-        <is>
-          <t>Joint</t>
-        </is>
-      </c>
-      <c r="D18" s="30" t="n">
-        <v>46311</v>
-      </c>
-      <c r="E18" s="30" t="n">
-        <v>46311</v>
-      </c>
-      <c r="F18" s="27">
+      <c r="A18" s="21" t="inlineStr">
+        <is>
+          <t>2.1</t>
+        </is>
+      </c>
+      <c r="B18" s="22" t="inlineStr">
+        <is>
+          <t>Rulebase hygiene analysis (shadowed, unused, any/any, overly permissive)</t>
+        </is>
+      </c>
+      <c r="C18" s="23" t="inlineStr">
+        <is>
+          <t>Consultant</t>
+        </is>
+      </c>
+      <c r="D18" s="24" t="n">
+        <v>46288</v>
+      </c>
+      <c r="E18" s="24" t="n">
+        <v>46294</v>
+      </c>
+      <c r="F18" s="21">
         <f>NETWORKDAYS(D18,E18,Inputs!$A$16:$A$21)</f>
         <v/>
       </c>
-      <c r="G18" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="H18" s="27">
+      <c r="G18" s="25" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H18" s="21">
         <f>IF(G18&gt;=1,"Complete",IF(E18&lt;Inputs!$B$7,"Late",IF(G18&gt;0,"In Progress",IF(D18&lt;=Inputs!$B$7,"Late Start","Not Started"))))</f>
         <v/>
       </c>
-      <c r="I18" s="29" t="inlineStr">
-        <is>
-          <t>1.7</t>
-        </is>
-      </c>
-      <c r="J18" s="32" t="inlineStr">
-        <is>
-          <t>Signed-off D1</t>
-        </is>
-      </c>
-      <c r="K18" s="32" t="inlineStr"/>
+      <c r="I18" s="23" t="inlineStr">
+        <is>
+          <t>1.3</t>
+        </is>
+      </c>
+      <c r="J18" s="26" t="inlineStr"/>
+      <c r="K18" s="26" t="inlineStr"/>
       <c r="L18" s="20" t="n"/>
       <c r="M18" s="20" t="n"/>
       <c r="N18" s="20" t="n"/>
@@ -2120,40 +2163,45 @@
       <c r="AA18" s="20" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="17" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="B19" s="3" t="inlineStr">
-        <is>
-          <t>Phase 2 – Identify Pain Points, Issues &amp; Gaps</t>
-        </is>
-      </c>
-      <c r="C19" s="17" t="inlineStr"/>
-      <c r="D19" s="18">
-        <f>MIN(D20:D26)</f>
-        <v/>
-      </c>
-      <c r="E19" s="18">
-        <f>MAX(E20:E26)</f>
-        <v/>
-      </c>
-      <c r="F19" s="17">
+      <c r="A19" s="21" t="inlineStr">
+        <is>
+          <t>2.2</t>
+        </is>
+      </c>
+      <c r="B19" s="22" t="inlineStr">
+        <is>
+          <t>NGFW feature utilization review (App-ID, User-ID, TLS decryption, IPS, URL, sandboxing)</t>
+        </is>
+      </c>
+      <c r="C19" s="23" t="inlineStr">
+        <is>
+          <t>Consultant</t>
+        </is>
+      </c>
+      <c r="D19" s="24" t="n">
+        <v>46288</v>
+      </c>
+      <c r="E19" s="24" t="n">
+        <v>46294</v>
+      </c>
+      <c r="F19" s="21">
         <f>NETWORKDAYS(D19,E19,Inputs!$A$16:$A$21)</f>
         <v/>
       </c>
-      <c r="G19" s="19">
-        <f>IFERROR(SUMPRODUCT(F20:F26,G20:G26)/SUM(F20:F26),0)</f>
-        <v/>
-      </c>
-      <c r="H19" s="17">
-        <f>IF(G19&gt;=1,"Complete",IF(G19&gt;0,"In Progress","Not Started"))</f>
-        <v/>
-      </c>
-      <c r="I19" s="17" t="n"/>
-      <c r="J19" s="3" t="n"/>
-      <c r="K19" s="3" t="n"/>
+      <c r="G19" s="25" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H19" s="21">
+        <f>IF(G19&gt;=1,"Complete",IF(E19&lt;Inputs!$B$7,"Late",IF(G19&gt;0,"In Progress",IF(D19&lt;=Inputs!$B$7,"Late Start","Not Started"))))</f>
+        <v/>
+      </c>
+      <c r="I19" s="23" t="inlineStr">
+        <is>
+          <t>1.3</t>
+        </is>
+      </c>
+      <c r="J19" s="26" t="inlineStr"/>
+      <c r="K19" s="26" t="inlineStr"/>
       <c r="L19" s="20" t="n"/>
       <c r="M19" s="20" t="n"/>
       <c r="N19" s="20" t="n"/>
@@ -2174,12 +2222,12 @@
     <row r="20">
       <c r="A20" s="21" t="inlineStr">
         <is>
-          <t>2.1</t>
+          <t>2.3</t>
         </is>
       </c>
       <c r="B20" s="22" t="inlineStr">
         <is>
-          <t>Rulebase hygiene analysis (shadowed, unused, any/any, overly permissive)</t>
+          <t>Maturity scoring (NIST CSF / CIS / vendor best practice) &amp; lifecycle risk review</t>
         </is>
       </c>
       <c r="C20" s="23" t="inlineStr">
@@ -2188,17 +2236,17 @@
         </is>
       </c>
       <c r="D20" s="24" t="n">
-        <v>46308</v>
+        <v>46293</v>
       </c>
       <c r="E20" s="24" t="n">
-        <v>46318</v>
+        <v>46296</v>
       </c>
       <c r="F20" s="21">
         <f>NETWORKDAYS(D20,E20,Inputs!$A$16:$A$21)</f>
         <v/>
       </c>
       <c r="G20" s="25" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="H20" s="21">
         <f>IF(G20&gt;=1,"Complete",IF(E20&lt;Inputs!$B$7,"Late",IF(G20&gt;0,"In Progress",IF(D20&lt;=Inputs!$B$7,"Late Start","Not Started"))))</f>
@@ -2206,10 +2254,14 @@
       </c>
       <c r="I20" s="23" t="inlineStr">
         <is>
-          <t>1.3</t>
-        </is>
-      </c>
-      <c r="J20" s="26" t="inlineStr"/>
+          <t>1.6</t>
+        </is>
+      </c>
+      <c r="J20" s="26" t="inlineStr">
+        <is>
+          <t>Maturity scorecard</t>
+        </is>
+      </c>
       <c r="K20" s="26" t="inlineStr"/>
       <c r="L20" s="20" t="n"/>
       <c r="M20" s="20" t="n"/>
@@ -2231,24 +2283,24 @@
     <row r="21">
       <c r="A21" s="21" t="inlineStr">
         <is>
-          <t>2.2</t>
+          <t>2.4</t>
         </is>
       </c>
       <c r="B21" s="22" t="inlineStr">
         <is>
-          <t>NGFW feature utilization review (App-ID, User-ID, TLS decryption, IPS, URL, sandboxing)</t>
+          <t>Gap &amp; pain-point validation workshop</t>
         </is>
       </c>
       <c r="C21" s="23" t="inlineStr">
         <is>
-          <t>Consultant</t>
+          <t>Joint</t>
         </is>
       </c>
       <c r="D21" s="24" t="n">
-        <v>46308</v>
+        <v>46296</v>
       </c>
       <c r="E21" s="24" t="n">
-        <v>46318</v>
+        <v>46296</v>
       </c>
       <c r="F21" s="21">
         <f>NETWORKDAYS(D21,E21,Inputs!$A$16:$A$21)</f>
@@ -2263,10 +2315,14 @@
       </c>
       <c r="I21" s="23" t="inlineStr">
         <is>
-          <t>1.3</t>
-        </is>
-      </c>
-      <c r="J21" s="26" t="inlineStr"/>
+          <t>2.3</t>
+        </is>
+      </c>
+      <c r="J21" s="26" t="inlineStr">
+        <is>
+          <t>Workshop output</t>
+        </is>
+      </c>
       <c r="K21" s="26" t="inlineStr"/>
       <c r="L21" s="20" t="n"/>
       <c r="M21" s="20" t="n"/>
@@ -2286,49 +2342,49 @@
       <c r="AA21" s="20" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="21" t="inlineStr">
-        <is>
-          <t>2.3</t>
-        </is>
-      </c>
-      <c r="B22" s="22" t="inlineStr">
-        <is>
-          <t>Maturity scoring vs. framework (NIST CSF / CIS / vendor best practice)</t>
-        </is>
-      </c>
-      <c r="C22" s="23" t="inlineStr">
+      <c r="A22" s="27" t="inlineStr">
+        <is>
+          <t>2.5</t>
+        </is>
+      </c>
+      <c r="B22" s="28" t="inlineStr">
+        <is>
+          <t>DELIVERABLE: Problem Areas &amp; Gaps Assessment document</t>
+        </is>
+      </c>
+      <c r="C22" s="29" t="inlineStr">
         <is>
           <t>Consultant</t>
         </is>
       </c>
-      <c r="D22" s="24" t="n">
-        <v>46314</v>
-      </c>
-      <c r="E22" s="24" t="n">
-        <v>46323</v>
-      </c>
-      <c r="F22" s="21">
+      <c r="D22" s="30" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E22" s="30" t="n">
+        <v>46297</v>
+      </c>
+      <c r="F22" s="27">
         <f>NETWORKDAYS(D22,E22,Inputs!$A$16:$A$21)</f>
         <v/>
       </c>
-      <c r="G22" s="25" t="n">
+      <c r="G22" s="31" t="n">
         <v>0</v>
       </c>
-      <c r="H22" s="21">
+      <c r="H22" s="27">
         <f>IF(G22&gt;=1,"Complete",IF(E22&lt;Inputs!$B$7,"Late",IF(G22&gt;0,"In Progress",IF(D22&lt;=Inputs!$B$7,"Late Start","Not Started"))))</f>
         <v/>
       </c>
-      <c r="I22" s="23" t="inlineStr">
-        <is>
-          <t>1.8</t>
-        </is>
-      </c>
-      <c r="J22" s="26" t="inlineStr">
-        <is>
-          <t>Maturity scorecard</t>
-        </is>
-      </c>
-      <c r="K22" s="26" t="inlineStr"/>
+      <c r="I22" s="29" t="inlineStr">
+        <is>
+          <t>2.4</t>
+        </is>
+      </c>
+      <c r="J22" s="32" t="inlineStr">
+        <is>
+          <t>D2 – Gaps Assessment</t>
+        </is>
+      </c>
+      <c r="K22" s="32" t="inlineStr"/>
       <c r="L22" s="20" t="n"/>
       <c r="M22" s="20" t="n"/>
       <c r="N22" s="20" t="n"/>
@@ -2347,45 +2403,40 @@
       <c r="AA22" s="20" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="21" t="inlineStr">
-        <is>
-          <t>2.4</t>
-        </is>
-      </c>
-      <c r="B23" s="22" t="inlineStr">
-        <is>
-          <t>Lifecycle, capacity &amp; resiliency risk review</t>
-        </is>
-      </c>
-      <c r="C23" s="23" t="inlineStr">
-        <is>
-          <t>Consultant</t>
-        </is>
-      </c>
-      <c r="D23" s="24" t="n">
-        <v>46314</v>
-      </c>
-      <c r="E23" s="24" t="n">
-        <v>46323</v>
-      </c>
-      <c r="F23" s="21">
+      <c r="A23" s="17" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Phase 3 – Define Future State Vision</t>
+        </is>
+      </c>
+      <c r="C23" s="17" t="inlineStr"/>
+      <c r="D23" s="18">
+        <f>MIN(D24:D26)</f>
+        <v/>
+      </c>
+      <c r="E23" s="18">
+        <f>MAX(E24:E26)</f>
+        <v/>
+      </c>
+      <c r="F23" s="17">
         <f>NETWORKDAYS(D23,E23,Inputs!$A$16:$A$21)</f>
         <v/>
       </c>
-      <c r="G23" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="H23" s="21">
-        <f>IF(G23&gt;=1,"Complete",IF(E23&lt;Inputs!$B$7,"Late",IF(G23&gt;0,"In Progress",IF(D23&lt;=Inputs!$B$7,"Late Start","Not Started"))))</f>
-        <v/>
-      </c>
-      <c r="I23" s="23" t="inlineStr">
-        <is>
-          <t>1.2</t>
-        </is>
-      </c>
-      <c r="J23" s="26" t="inlineStr"/>
-      <c r="K23" s="26" t="inlineStr"/>
+      <c r="G23" s="19">
+        <f>IFERROR(SUMPRODUCT(F24:F26,G24:G26)/SUM(F24:F26),0)</f>
+        <v/>
+      </c>
+      <c r="H23" s="17">
+        <f>IF(G23&gt;=1,"Complete",IF(G23&gt;0,"In Progress","Not Started"))</f>
+        <v/>
+      </c>
+      <c r="I23" s="17" t="n"/>
+      <c r="J23" s="3" t="n"/>
+      <c r="K23" s="3" t="n"/>
       <c r="L23" s="20" t="n"/>
       <c r="M23" s="20" t="n"/>
       <c r="N23" s="20" t="n"/>
@@ -2406,24 +2457,24 @@
     <row r="24">
       <c r="A24" s="21" t="inlineStr">
         <is>
-          <t>2.5</t>
+          <t>3.1</t>
         </is>
       </c>
       <c r="B24" s="22" t="inlineStr">
         <is>
-          <t>Gap &amp; pain-point validation workshop</t>
+          <t>Requirements, guiding principles &amp; target architecture options</t>
         </is>
       </c>
       <c r="C24" s="23" t="inlineStr">
         <is>
-          <t>Joint</t>
+          <t>Consultant</t>
         </is>
       </c>
       <c r="D24" s="24" t="n">
-        <v>46324</v>
+        <v>46295</v>
       </c>
       <c r="E24" s="24" t="n">
-        <v>46325</v>
+        <v>46297</v>
       </c>
       <c r="F24" s="21">
         <f>NETWORKDAYS(D24,E24,Inputs!$A$16:$A$21)</f>
@@ -2438,12 +2489,12 @@
       </c>
       <c r="I24" s="23" t="inlineStr">
         <is>
-          <t>2.3</t>
+          <t>2.4</t>
         </is>
       </c>
       <c r="J24" s="26" t="inlineStr">
         <is>
-          <t>Workshop output</t>
+          <t>Options analysis</t>
         </is>
       </c>
       <c r="K24" s="26" t="inlineStr"/>
@@ -2465,49 +2516,49 @@
       <c r="AA24" s="20" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="27" t="inlineStr">
-        <is>
-          <t>2.6</t>
-        </is>
-      </c>
-      <c r="B25" s="28" t="inlineStr">
-        <is>
-          <t>DELIVERABLE: Problem Areas &amp; Gaps Assessment document</t>
-        </is>
-      </c>
-      <c r="C25" s="29" t="inlineStr">
-        <is>
-          <t>Consultant</t>
-        </is>
-      </c>
-      <c r="D25" s="30" t="n">
-        <v>46328</v>
-      </c>
-      <c r="E25" s="30" t="n">
-        <v>46332</v>
-      </c>
-      <c r="F25" s="27">
+      <c r="A25" s="21" t="inlineStr">
+        <is>
+          <t>3.2</t>
+        </is>
+      </c>
+      <c r="B25" s="22" t="inlineStr">
+        <is>
+          <t>Future-state vision workshop &amp; option selection</t>
+        </is>
+      </c>
+      <c r="C25" s="23" t="inlineStr">
+        <is>
+          <t>Joint</t>
+        </is>
+      </c>
+      <c r="D25" s="24" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E25" s="24" t="n">
+        <v>46300</v>
+      </c>
+      <c r="F25" s="21">
         <f>NETWORKDAYS(D25,E25,Inputs!$A$16:$A$21)</f>
         <v/>
       </c>
-      <c r="G25" s="31" t="n">
+      <c r="G25" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H25" s="27">
+      <c r="H25" s="21">
         <f>IF(G25&gt;=1,"Complete",IF(E25&lt;Inputs!$B$7,"Late",IF(G25&gt;0,"In Progress",IF(D25&lt;=Inputs!$B$7,"Late Start","Not Started"))))</f>
         <v/>
       </c>
-      <c r="I25" s="29" t="inlineStr">
-        <is>
-          <t>2.5</t>
-        </is>
-      </c>
-      <c r="J25" s="32" t="inlineStr">
-        <is>
-          <t>D2 – Gaps Assessment</t>
-        </is>
-      </c>
-      <c r="K25" s="32" t="inlineStr"/>
+      <c r="I25" s="23" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
+      </c>
+      <c r="J25" s="26" t="inlineStr">
+        <is>
+          <t>Decision log</t>
+        </is>
+      </c>
+      <c r="K25" s="26" t="inlineStr"/>
       <c r="L25" s="20" t="n"/>
       <c r="M25" s="20" t="n"/>
       <c r="N25" s="20" t="n"/>
@@ -2526,49 +2577,49 @@
       <c r="AA25" s="20" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="27" t="inlineStr">
-        <is>
-          <t>2.7</t>
-        </is>
-      </c>
-      <c r="B26" s="33" t="inlineStr">
-        <is>
-          <t>Milestone: Gaps Assessment accepted</t>
-        </is>
-      </c>
-      <c r="C26" s="29" t="inlineStr">
-        <is>
-          <t>Joint</t>
-        </is>
-      </c>
-      <c r="D26" s="30" t="n">
-        <v>46332</v>
-      </c>
-      <c r="E26" s="30" t="n">
-        <v>46332</v>
-      </c>
-      <c r="F26" s="27">
+      <c r="A26" s="21" t="inlineStr">
+        <is>
+          <t>3.3</t>
+        </is>
+      </c>
+      <c r="B26" s="22" t="inlineStr">
+        <is>
+          <t>Future-state architecture, target operating model &amp; maturity targets</t>
+        </is>
+      </c>
+      <c r="C26" s="23" t="inlineStr">
+        <is>
+          <t>Consultant</t>
+        </is>
+      </c>
+      <c r="D26" s="24" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E26" s="24" t="n">
+        <v>46301</v>
+      </c>
+      <c r="F26" s="21">
         <f>NETWORKDAYS(D26,E26,Inputs!$A$16:$A$21)</f>
         <v/>
       </c>
-      <c r="G26" s="31" t="n">
+      <c r="G26" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H26" s="27">
+      <c r="H26" s="21">
         <f>IF(G26&gt;=1,"Complete",IF(E26&lt;Inputs!$B$7,"Late",IF(G26&gt;0,"In Progress",IF(D26&lt;=Inputs!$B$7,"Late Start","Not Started"))))</f>
         <v/>
       </c>
-      <c r="I26" s="29" t="inlineStr">
-        <is>
-          <t>2.6</t>
-        </is>
-      </c>
-      <c r="J26" s="32" t="inlineStr">
-        <is>
-          <t>Signed-off D2</t>
-        </is>
-      </c>
-      <c r="K26" s="32" t="inlineStr"/>
+      <c r="I26" s="23" t="inlineStr">
+        <is>
+          <t>3.2</t>
+        </is>
+      </c>
+      <c r="J26" s="26" t="inlineStr">
+        <is>
+          <t>Future-state architecture</t>
+        </is>
+      </c>
+      <c r="K26" s="26" t="inlineStr"/>
       <c r="L26" s="20" t="n"/>
       <c r="M26" s="20" t="n"/>
       <c r="N26" s="20" t="n"/>
@@ -2589,21 +2640,21 @@
     <row r="27">
       <c r="A27" s="17" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>Phase 3 – Define Future State Vision</t>
+          <t>Phase 4 – Remediation Plan &amp; Modernization Roadmap</t>
         </is>
       </c>
       <c r="C27" s="17" t="inlineStr"/>
       <c r="D27" s="18">
-        <f>MIN(D28:D33)</f>
+        <f>MIN(D28:D30)</f>
         <v/>
       </c>
       <c r="E27" s="18">
-        <f>MAX(E28:E33)</f>
+        <f>MAX(E28:E30)</f>
         <v/>
       </c>
       <c r="F27" s="17">
@@ -2611,7 +2662,7 @@
         <v/>
       </c>
       <c r="G27" s="19">
-        <f>IFERROR(SUMPRODUCT(F28:F33,G28:G33)/SUM(F28:F33),0)</f>
+        <f>IFERROR(SUMPRODUCT(F28:F30,G28:G30)/SUM(F28:F30),0)</f>
         <v/>
       </c>
       <c r="H27" s="17">
@@ -2641,12 +2692,12 @@
     <row r="28">
       <c r="A28" s="21" t="inlineStr">
         <is>
-          <t>3.1</t>
+          <t>4.1</t>
         </is>
       </c>
       <c r="B28" s="22" t="inlineStr">
         <is>
-          <t>Business &amp; security requirements / guiding principles</t>
+          <t>Gap-to-initiative mapping, prioritization &amp; sequencing</t>
         </is>
       </c>
       <c r="C28" s="23" t="inlineStr">
@@ -2655,10 +2706,10 @@
         </is>
       </c>
       <c r="D28" s="24" t="n">
-        <v>46328</v>
+        <v>46300</v>
       </c>
       <c r="E28" s="24" t="n">
-        <v>46332</v>
+        <v>46302</v>
       </c>
       <c r="F28" s="21">
         <f>NETWORKDAYS(D28,E28,Inputs!$A$16:$A$21)</f>
@@ -2673,10 +2724,14 @@
       </c>
       <c r="I28" s="23" t="inlineStr">
         <is>
-          <t>2.5</t>
-        </is>
-      </c>
-      <c r="J28" s="26" t="inlineStr"/>
+          <t>3.2</t>
+        </is>
+      </c>
+      <c r="J28" s="26" t="inlineStr">
+        <is>
+          <t>Prioritization matrix</t>
+        </is>
+      </c>
       <c r="K28" s="26" t="inlineStr"/>
       <c r="L28" s="20" t="n"/>
       <c r="M28" s="20" t="n"/>
@@ -2696,49 +2751,49 @@
       <c r="AA28" s="20" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="21" t="inlineStr">
-        <is>
-          <t>3.2</t>
-        </is>
-      </c>
-      <c r="B29" s="22" t="inlineStr">
-        <is>
-          <t>Target architecture options (consolidation, platform, cloud/SASE, zero trust segmentation)</t>
-        </is>
-      </c>
-      <c r="C29" s="23" t="inlineStr">
+      <c r="A29" s="27" t="inlineStr">
+        <is>
+          <t>4.2</t>
+        </is>
+      </c>
+      <c r="B29" s="28" t="inlineStr">
+        <is>
+          <t>DELIVERABLE: Modernization Roadmap (incl. remediation plan)</t>
+        </is>
+      </c>
+      <c r="C29" s="29" t="inlineStr">
         <is>
           <t>Consultant</t>
         </is>
       </c>
-      <c r="D29" s="24" t="n">
-        <v>46335</v>
-      </c>
-      <c r="E29" s="24" t="n">
-        <v>46344</v>
-      </c>
-      <c r="F29" s="21">
+      <c r="D29" s="30" t="n">
+        <v>46302</v>
+      </c>
+      <c r="E29" s="30" t="n">
+        <v>46303</v>
+      </c>
+      <c r="F29" s="27">
         <f>NETWORKDAYS(D29,E29,Inputs!$A$16:$A$21)</f>
         <v/>
       </c>
-      <c r="G29" s="25" t="n">
+      <c r="G29" s="31" t="n">
         <v>0</v>
       </c>
-      <c r="H29" s="21">
+      <c r="H29" s="27">
         <f>IF(G29&gt;=1,"Complete",IF(E29&lt;Inputs!$B$7,"Late",IF(G29&gt;0,"In Progress",IF(D29&lt;=Inputs!$B$7,"Late Start","Not Started"))))</f>
         <v/>
       </c>
-      <c r="I29" s="23" t="inlineStr">
-        <is>
-          <t>3.1</t>
-        </is>
-      </c>
-      <c r="J29" s="26" t="inlineStr">
-        <is>
-          <t>Options analysis</t>
-        </is>
-      </c>
-      <c r="K29" s="26" t="inlineStr"/>
+      <c r="I29" s="29" t="inlineStr">
+        <is>
+          <t>4.1</t>
+        </is>
+      </c>
+      <c r="J29" s="32" t="inlineStr">
+        <is>
+          <t>D3 – Modernization Roadmap</t>
+        </is>
+      </c>
+      <c r="K29" s="32" t="inlineStr"/>
       <c r="L29" s="20" t="n"/>
       <c r="M29" s="20" t="n"/>
       <c r="N29" s="20" t="n"/>
@@ -2757,45 +2812,49 @@
       <c r="AA29" s="20" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="21" t="inlineStr">
-        <is>
-          <t>3.3</t>
-        </is>
-      </c>
-      <c r="B30" s="22" t="inlineStr">
-        <is>
-          <t>Target operating model (policy lifecycle, automation, ownership)</t>
-        </is>
-      </c>
-      <c r="C30" s="23" t="inlineStr">
-        <is>
-          <t>Consultant</t>
-        </is>
-      </c>
-      <c r="D30" s="24" t="n">
-        <v>46335</v>
-      </c>
-      <c r="E30" s="24" t="n">
-        <v>46344</v>
-      </c>
-      <c r="F30" s="21">
+      <c r="A30" s="27" t="inlineStr">
+        <is>
+          <t>4.3</t>
+        </is>
+      </c>
+      <c r="B30" s="33" t="inlineStr">
+        <is>
+          <t>Milestone: Executive readout – D1, D2, D3 presented &amp; accepted</t>
+        </is>
+      </c>
+      <c r="C30" s="29" t="inlineStr">
+        <is>
+          <t>Joint</t>
+        </is>
+      </c>
+      <c r="D30" s="30" t="n">
+        <v>46304</v>
+      </c>
+      <c r="E30" s="30" t="n">
+        <v>46304</v>
+      </c>
+      <c r="F30" s="27">
         <f>NETWORKDAYS(D30,E30,Inputs!$A$16:$A$21)</f>
         <v/>
       </c>
-      <c r="G30" s="25" t="n">
+      <c r="G30" s="31" t="n">
         <v>0</v>
       </c>
-      <c r="H30" s="21">
+      <c r="H30" s="27">
         <f>IF(G30&gt;=1,"Complete",IF(E30&lt;Inputs!$B$7,"Late",IF(G30&gt;0,"In Progress",IF(D30&lt;=Inputs!$B$7,"Late Start","Not Started"))))</f>
         <v/>
       </c>
-      <c r="I30" s="23" t="inlineStr">
-        <is>
-          <t>3.1</t>
-        </is>
-      </c>
-      <c r="J30" s="26" t="inlineStr"/>
-      <c r="K30" s="26" t="inlineStr"/>
+      <c r="I30" s="29" t="inlineStr">
+        <is>
+          <t>4.2</t>
+        </is>
+      </c>
+      <c r="J30" s="32" t="inlineStr">
+        <is>
+          <t>Executive readout deck</t>
+        </is>
+      </c>
+      <c r="K30" s="32" t="inlineStr"/>
       <c r="L30" s="20" t="n"/>
       <c r="M30" s="20" t="n"/>
       <c r="N30" s="20" t="n"/>
@@ -2814,49 +2873,40 @@
       <c r="AA30" s="20" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="21" t="inlineStr">
-        <is>
-          <t>3.4</t>
-        </is>
-      </c>
-      <c r="B31" s="22" t="inlineStr">
-        <is>
-          <t>Future-state vision workshop &amp; option selection</t>
-        </is>
-      </c>
-      <c r="C31" s="23" t="inlineStr">
-        <is>
-          <t>Joint</t>
-        </is>
-      </c>
-      <c r="D31" s="24" t="n">
-        <v>46345</v>
-      </c>
-      <c r="E31" s="24" t="n">
-        <v>46346</v>
-      </c>
-      <c r="F31" s="21">
+      <c r="A31" s="17" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>Phase 5 – Remediation Mobilization</t>
+        </is>
+      </c>
+      <c r="C31" s="17" t="inlineStr"/>
+      <c r="D31" s="18">
+        <f>MIN(D32:D34)</f>
+        <v/>
+      </c>
+      <c r="E31" s="18">
+        <f>MAX(E32:E34)</f>
+        <v/>
+      </c>
+      <c r="F31" s="17">
         <f>NETWORKDAYS(D31,E31,Inputs!$A$16:$A$21)</f>
         <v/>
       </c>
-      <c r="G31" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="H31" s="21">
-        <f>IF(G31&gt;=1,"Complete",IF(E31&lt;Inputs!$B$7,"Late",IF(G31&gt;0,"In Progress",IF(D31&lt;=Inputs!$B$7,"Late Start","Not Started"))))</f>
-        <v/>
-      </c>
-      <c r="I31" s="23" t="inlineStr">
-        <is>
-          <t>3.2</t>
-        </is>
-      </c>
-      <c r="J31" s="26" t="inlineStr">
-        <is>
-          <t>Decision log</t>
-        </is>
-      </c>
-      <c r="K31" s="26" t="inlineStr"/>
+      <c r="G31" s="19">
+        <f>IFERROR(SUMPRODUCT(F32:F34,G32:G34)/SUM(F32:F34),0)</f>
+        <v/>
+      </c>
+      <c r="H31" s="17">
+        <f>IF(G31&gt;=1,"Complete",IF(G31&gt;0,"In Progress","Not Started"))</f>
+        <v/>
+      </c>
+      <c r="I31" s="17" t="n"/>
+      <c r="J31" s="3" t="n"/>
+      <c r="K31" s="3" t="n"/>
       <c r="L31" s="20" t="n"/>
       <c r="M31" s="20" t="n"/>
       <c r="N31" s="20" t="n"/>
@@ -2877,24 +2927,24 @@
     <row r="32">
       <c r="A32" s="21" t="inlineStr">
         <is>
-          <t>3.5</t>
+          <t>5.1</t>
         </is>
       </c>
       <c r="B32" s="22" t="inlineStr">
         <is>
-          <t>Future-state architecture &amp; target maturity levels documented</t>
+          <t>Detailed remediation work plan, change windows &amp; CAB scheduling</t>
         </is>
       </c>
       <c r="C32" s="23" t="inlineStr">
         <is>
-          <t>Consultant</t>
+          <t>Joint</t>
         </is>
       </c>
       <c r="D32" s="24" t="n">
-        <v>46349</v>
+        <v>46308</v>
       </c>
       <c r="E32" s="24" t="n">
-        <v>46351</v>
+        <v>46310</v>
       </c>
       <c r="F32" s="21">
         <f>NETWORKDAYS(D32,E32,Inputs!$A$16:$A$21)</f>
@@ -2909,12 +2959,12 @@
       </c>
       <c r="I32" s="23" t="inlineStr">
         <is>
-          <t>3.4</t>
+          <t>4.3</t>
         </is>
       </c>
       <c r="J32" s="26" t="inlineStr">
         <is>
-          <t>Future-state architecture</t>
+          <t>D4 – Remediation Execution Plan</t>
         </is>
       </c>
       <c r="K32" s="26" t="inlineStr"/>
@@ -2936,45 +2986,49 @@
       <c r="AA32" s="20" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="27" t="inlineStr">
-        <is>
-          <t>3.6</t>
-        </is>
-      </c>
-      <c r="B33" s="33" t="inlineStr">
-        <is>
-          <t>Milestone: Future-state vision approved</t>
-        </is>
-      </c>
-      <c r="C33" s="29" t="inlineStr">
-        <is>
-          <t>Joint</t>
-        </is>
-      </c>
-      <c r="D33" s="30" t="n">
-        <v>46351</v>
-      </c>
-      <c r="E33" s="30" t="n">
-        <v>46351</v>
-      </c>
-      <c r="F33" s="27">
+      <c r="A33" s="21" t="inlineStr">
+        <is>
+          <t>5.2</t>
+        </is>
+      </c>
+      <c r="B33" s="22" t="inlineStr">
+        <is>
+          <t>Config backups, rollback procedures &amp; test / validation plans</t>
+        </is>
+      </c>
+      <c r="C33" s="23" t="inlineStr">
+        <is>
+          <t>Consultant</t>
+        </is>
+      </c>
+      <c r="D33" s="24" t="n">
+        <v>46308</v>
+      </c>
+      <c r="E33" s="24" t="n">
+        <v>46311</v>
+      </c>
+      <c r="F33" s="21">
         <f>NETWORKDAYS(D33,E33,Inputs!$A$16:$A$21)</f>
         <v/>
       </c>
-      <c r="G33" s="31" t="n">
+      <c r="G33" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H33" s="27">
+      <c r="H33" s="21">
         <f>IF(G33&gt;=1,"Complete",IF(E33&lt;Inputs!$B$7,"Late",IF(G33&gt;0,"In Progress",IF(D33&lt;=Inputs!$B$7,"Late Start","Not Started"))))</f>
         <v/>
       </c>
-      <c r="I33" s="29" t="inlineStr">
-        <is>
-          <t>3.5</t>
-        </is>
-      </c>
-      <c r="J33" s="32" t="inlineStr"/>
-      <c r="K33" s="32" t="inlineStr"/>
+      <c r="I33" s="23" t="inlineStr">
+        <is>
+          <t>4.3</t>
+        </is>
+      </c>
+      <c r="J33" s="26" t="inlineStr">
+        <is>
+          <t>Rollback &amp; test plans</t>
+        </is>
+      </c>
+      <c r="K33" s="26" t="inlineStr"/>
       <c r="L33" s="20" t="n"/>
       <c r="M33" s="20" t="n"/>
       <c r="N33" s="20" t="n"/>
@@ -2993,40 +3047,45 @@
       <c r="AA33" s="20" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="17" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="B34" s="3" t="inlineStr">
-        <is>
-          <t>Phase 4 – Remediation Plan &amp; Modernization Roadmap</t>
-        </is>
-      </c>
-      <c r="C34" s="17" t="inlineStr"/>
-      <c r="D34" s="18">
-        <f>MIN(D35:D39)</f>
-        <v/>
-      </c>
-      <c r="E34" s="18">
-        <f>MAX(E35:E39)</f>
-        <v/>
-      </c>
-      <c r="F34" s="17">
+      <c r="A34" s="27" t="inlineStr">
+        <is>
+          <t>5.3</t>
+        </is>
+      </c>
+      <c r="B34" s="33" t="inlineStr">
+        <is>
+          <t>Milestone: Remediation go / no-go</t>
+        </is>
+      </c>
+      <c r="C34" s="29" t="inlineStr">
+        <is>
+          <t>Joint</t>
+        </is>
+      </c>
+      <c r="D34" s="30" t="n">
+        <v>46311</v>
+      </c>
+      <c r="E34" s="30" t="n">
+        <v>46311</v>
+      </c>
+      <c r="F34" s="27">
         <f>NETWORKDAYS(D34,E34,Inputs!$A$16:$A$21)</f>
         <v/>
       </c>
-      <c r="G34" s="19">
-        <f>IFERROR(SUMPRODUCT(F35:F39,G35:G39)/SUM(F35:F39),0)</f>
-        <v/>
-      </c>
-      <c r="H34" s="17">
-        <f>IF(G34&gt;=1,"Complete",IF(G34&gt;0,"In Progress","Not Started"))</f>
-        <v/>
-      </c>
-      <c r="I34" s="17" t="n"/>
-      <c r="J34" s="3" t="n"/>
-      <c r="K34" s="3" t="n"/>
+      <c r="G34" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="H34" s="27">
+        <f>IF(G34&gt;=1,"Complete",IF(E34&lt;Inputs!$B$7,"Late",IF(G34&gt;0,"In Progress",IF(D34&lt;=Inputs!$B$7,"Late Start","Not Started"))))</f>
+        <v/>
+      </c>
+      <c r="I34" s="29" t="inlineStr">
+        <is>
+          <t>5.1</t>
+        </is>
+      </c>
+      <c r="J34" s="32" t="inlineStr"/>
+      <c r="K34" s="32" t="inlineStr"/>
       <c r="L34" s="20" t="n"/>
       <c r="M34" s="20" t="n"/>
       <c r="N34" s="20" t="n"/>
@@ -3045,49 +3104,40 @@
       <c r="AA34" s="20" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="21" t="inlineStr">
-        <is>
-          <t>4.1</t>
-        </is>
-      </c>
-      <c r="B35" s="22" t="inlineStr">
-        <is>
-          <t>Gap-to-initiative mapping &amp; quick wins</t>
-        </is>
-      </c>
-      <c r="C35" s="23" t="inlineStr">
-        <is>
-          <t>Consultant</t>
-        </is>
-      </c>
-      <c r="D35" s="24" t="n">
-        <v>46356</v>
-      </c>
-      <c r="E35" s="24" t="n">
-        <v>46360</v>
-      </c>
-      <c r="F35" s="21">
+      <c r="A35" s="17" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>Phase 6 – Remediation Execution</t>
+        </is>
+      </c>
+      <c r="C35" s="17" t="inlineStr"/>
+      <c r="D35" s="18">
+        <f>MIN(D36:D43)</f>
+        <v/>
+      </c>
+      <c r="E35" s="18">
+        <f>MAX(E36:E43)</f>
+        <v/>
+      </c>
+      <c r="F35" s="17">
         <f>NETWORKDAYS(D35,E35,Inputs!$A$16:$A$21)</f>
         <v/>
       </c>
-      <c r="G35" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="H35" s="21">
-        <f>IF(G35&gt;=1,"Complete",IF(E35&lt;Inputs!$B$7,"Late",IF(G35&gt;0,"In Progress",IF(D35&lt;=Inputs!$B$7,"Late Start","Not Started"))))</f>
-        <v/>
-      </c>
-      <c r="I35" s="23" t="inlineStr">
-        <is>
-          <t>3.6</t>
-        </is>
-      </c>
-      <c r="J35" s="26" t="inlineStr">
-        <is>
-          <t>Initiative catalog</t>
-        </is>
-      </c>
-      <c r="K35" s="26" t="inlineStr"/>
+      <c r="G35" s="19">
+        <f>IFERROR(SUMPRODUCT(F36:F43,G36:G43)/SUM(F36:F43),0)</f>
+        <v/>
+      </c>
+      <c r="H35" s="17">
+        <f>IF(G35&gt;=1,"Complete",IF(G35&gt;0,"In Progress","Not Started"))</f>
+        <v/>
+      </c>
+      <c r="I35" s="17" t="n"/>
+      <c r="J35" s="3" t="n"/>
+      <c r="K35" s="3" t="n"/>
       <c r="L35" s="20" t="n"/>
       <c r="M35" s="20" t="n"/>
       <c r="N35" s="20" t="n"/>
@@ -3108,12 +3158,12 @@
     <row r="36">
       <c r="A36" s="21" t="inlineStr">
         <is>
-          <t>4.2</t>
+          <t>6.1</t>
         </is>
       </c>
       <c r="B36" s="22" t="inlineStr">
         <is>
-          <t>Prioritization (risk reduction, effort, cost, dependencies)</t>
+          <t>Quick wins: rulebase cleanup (unused, shadowed, any/any, redundant objects)</t>
         </is>
       </c>
       <c r="C36" s="23" t="inlineStr">
@@ -3122,10 +3172,10 @@
         </is>
       </c>
       <c r="D36" s="24" t="n">
-        <v>46357</v>
+        <v>46314</v>
       </c>
       <c r="E36" s="24" t="n">
-        <v>46364</v>
+        <v>46332</v>
       </c>
       <c r="F36" s="21">
         <f>NETWORKDAYS(D36,E36,Inputs!$A$16:$A$21)</f>
@@ -3140,12 +3190,12 @@
       </c>
       <c r="I36" s="23" t="inlineStr">
         <is>
-          <t>4.1</t>
+          <t>5.3</t>
         </is>
       </c>
       <c r="J36" s="26" t="inlineStr">
         <is>
-          <t>Prioritization matrix</t>
+          <t>Cleanup change records</t>
         </is>
       </c>
       <c r="K36" s="26" t="inlineStr"/>
@@ -3169,24 +3219,24 @@
     <row r="37">
       <c r="A37" s="21" t="inlineStr">
         <is>
-          <t>4.3</t>
+          <t>6.2</t>
         </is>
       </c>
       <c r="B37" s="22" t="inlineStr">
         <is>
-          <t>Sequencing into horizons (0–6, 6–12, 12–24 months)</t>
+          <t>Software / firmware upgrades &amp; EoL/EoS hardware remediation</t>
         </is>
       </c>
       <c r="C37" s="23" t="inlineStr">
         <is>
-          <t>Consultant</t>
+          <t>Joint</t>
         </is>
       </c>
       <c r="D37" s="24" t="n">
-        <v>46363</v>
+        <v>46321</v>
       </c>
       <c r="E37" s="24" t="n">
-        <v>46367</v>
+        <v>46346</v>
       </c>
       <c r="F37" s="21">
         <f>NETWORKDAYS(D37,E37,Inputs!$A$16:$A$21)</f>
@@ -3201,10 +3251,14 @@
       </c>
       <c r="I37" s="23" t="inlineStr">
         <is>
-          <t>4.2</t>
-        </is>
-      </c>
-      <c r="J37" s="26" t="inlineStr"/>
+          <t>5.3</t>
+        </is>
+      </c>
+      <c r="J37" s="26" t="inlineStr">
+        <is>
+          <t>Upgrade change records</t>
+        </is>
+      </c>
       <c r="K37" s="26" t="inlineStr"/>
       <c r="L37" s="20" t="n"/>
       <c r="M37" s="20" t="n"/>
@@ -3226,12 +3280,12 @@
     <row r="38">
       <c r="A38" s="21" t="inlineStr">
         <is>
-          <t>4.4</t>
+          <t>6.3</t>
         </is>
       </c>
       <c r="B38" s="22" t="inlineStr">
         <is>
-          <t>High-level budget, resourcing &amp; success metrics / KPIs</t>
+          <t>Logging, SIEM integration &amp; monitoring / alerting tuning</t>
         </is>
       </c>
       <c r="C38" s="23" t="inlineStr">
@@ -3240,10 +3294,10 @@
         </is>
       </c>
       <c r="D38" s="24" t="n">
-        <v>46363</v>
+        <v>46321</v>
       </c>
       <c r="E38" s="24" t="n">
-        <v>46367</v>
+        <v>46339</v>
       </c>
       <c r="F38" s="21">
         <f>NETWORKDAYS(D38,E38,Inputs!$A$16:$A$21)</f>
@@ -3258,7 +3312,7 @@
       </c>
       <c r="I38" s="23" t="inlineStr">
         <is>
-          <t>4.2</t>
+          <t>5.3</t>
         </is>
       </c>
       <c r="J38" s="26" t="inlineStr"/>
@@ -3281,49 +3335,45 @@
       <c r="AA38" s="20" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="27" t="inlineStr">
-        <is>
-          <t>4.5</t>
-        </is>
-      </c>
-      <c r="B39" s="28" t="inlineStr">
-        <is>
-          <t>DELIVERABLE: Modernization Roadmap (incl. remediation plan)</t>
-        </is>
-      </c>
-      <c r="C39" s="29" t="inlineStr">
-        <is>
-          <t>Consultant</t>
-        </is>
-      </c>
-      <c r="D39" s="30" t="n">
-        <v>46367</v>
-      </c>
-      <c r="E39" s="30" t="n">
-        <v>46373</v>
-      </c>
-      <c r="F39" s="27">
+      <c r="A39" s="21" t="inlineStr">
+        <is>
+          <t>6.4</t>
+        </is>
+      </c>
+      <c r="B39" s="22" t="inlineStr">
+        <is>
+          <t>Enable NGFW security profiles (App-ID migration, User-ID, IPS, URL, sandboxing)</t>
+        </is>
+      </c>
+      <c r="C39" s="23" t="inlineStr">
+        <is>
+          <t>Joint</t>
+        </is>
+      </c>
+      <c r="D39" s="24" t="n">
+        <v>46328</v>
+      </c>
+      <c r="E39" s="24" t="n">
+        <v>46360</v>
+      </c>
+      <c r="F39" s="21">
         <f>NETWORKDAYS(D39,E39,Inputs!$A$16:$A$21)</f>
         <v/>
       </c>
-      <c r="G39" s="31" t="n">
+      <c r="G39" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H39" s="27">
+      <c r="H39" s="21">
         <f>IF(G39&gt;=1,"Complete",IF(E39&lt;Inputs!$B$7,"Late",IF(G39&gt;0,"In Progress",IF(D39&lt;=Inputs!$B$7,"Late Start","Not Started"))))</f>
         <v/>
       </c>
-      <c r="I39" s="29" t="inlineStr">
-        <is>
-          <t>4.3</t>
-        </is>
-      </c>
-      <c r="J39" s="32" t="inlineStr">
-        <is>
-          <t>D3 – Modernization Roadmap</t>
-        </is>
-      </c>
-      <c r="K39" s="32" t="inlineStr"/>
+      <c r="I39" s="23" t="inlineStr">
+        <is>
+          <t>6.1</t>
+        </is>
+      </c>
+      <c r="J39" s="26" t="inlineStr"/>
+      <c r="K39" s="26" t="inlineStr"/>
       <c r="L39" s="20" t="n"/>
       <c r="M39" s="20" t="n"/>
       <c r="N39" s="20" t="n"/>
@@ -3342,40 +3392,45 @@
       <c r="AA39" s="20" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="17" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="B40" s="3" t="inlineStr">
-        <is>
-          <t>Phase 5 – Executive Readout &amp; Closeout</t>
-        </is>
-      </c>
-      <c r="C40" s="17" t="inlineStr"/>
-      <c r="D40" s="18">
-        <f>MIN(D41:D44)</f>
-        <v/>
-      </c>
-      <c r="E40" s="18">
-        <f>MAX(E41:E44)</f>
-        <v/>
-      </c>
-      <c r="F40" s="17">
+      <c r="A40" s="21" t="inlineStr">
+        <is>
+          <t>6.5</t>
+        </is>
+      </c>
+      <c r="B40" s="22" t="inlineStr">
+        <is>
+          <t>Segmentation &amp; zone redesign (zero trust alignment)</t>
+        </is>
+      </c>
+      <c r="C40" s="23" t="inlineStr">
+        <is>
+          <t>Joint</t>
+        </is>
+      </c>
+      <c r="D40" s="24" t="n">
+        <v>46335</v>
+      </c>
+      <c r="E40" s="24" t="n">
+        <v>46367</v>
+      </c>
+      <c r="F40" s="21">
         <f>NETWORKDAYS(D40,E40,Inputs!$A$16:$A$21)</f>
         <v/>
       </c>
-      <c r="G40" s="19">
-        <f>IFERROR(SUMPRODUCT(F41:F44,G41:G44)/SUM(F41:F44),0)</f>
-        <v/>
-      </c>
-      <c r="H40" s="17">
-        <f>IF(G40&gt;=1,"Complete",IF(G40&gt;0,"In Progress","Not Started"))</f>
-        <v/>
-      </c>
-      <c r="I40" s="17" t="n"/>
-      <c r="J40" s="3" t="n"/>
-      <c r="K40" s="3" t="n"/>
+      <c r="G40" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H40" s="21">
+        <f>IF(G40&gt;=1,"Complete",IF(E40&lt;Inputs!$B$7,"Late",IF(G40&gt;0,"In Progress",IF(D40&lt;=Inputs!$B$7,"Late Start","Not Started"))))</f>
+        <v/>
+      </c>
+      <c r="I40" s="23" t="inlineStr">
+        <is>
+          <t>6.1</t>
+        </is>
+      </c>
+      <c r="J40" s="26" t="inlineStr"/>
+      <c r="K40" s="26" t="inlineStr"/>
       <c r="L40" s="20" t="n"/>
       <c r="M40" s="20" t="n"/>
       <c r="N40" s="20" t="n"/>
@@ -3396,12 +3451,12 @@
     <row r="41">
       <c r="A41" s="21" t="inlineStr">
         <is>
-          <t>5.1</t>
+          <t>6.6</t>
         </is>
       </c>
       <c r="B41" s="22" t="inlineStr">
         <is>
-          <t>Executive readout / steering committee presentation</t>
+          <t>Phased TLS/SSL decryption rollout</t>
         </is>
       </c>
       <c r="C41" s="23" t="inlineStr">
@@ -3410,10 +3465,10 @@
         </is>
       </c>
       <c r="D41" s="24" t="n">
-        <v>46374</v>
+        <v>46342</v>
       </c>
       <c r="E41" s="24" t="n">
-        <v>46374</v>
+        <v>46367</v>
       </c>
       <c r="F41" s="21">
         <f>NETWORKDAYS(D41,E41,Inputs!$A$16:$A$21)</f>
@@ -3428,14 +3483,10 @@
       </c>
       <c r="I41" s="23" t="inlineStr">
         <is>
-          <t>4.5</t>
-        </is>
-      </c>
-      <c r="J41" s="26" t="inlineStr">
-        <is>
-          <t>Executive readout deck</t>
-        </is>
-      </c>
+          <t>6.4</t>
+        </is>
+      </c>
+      <c r="J41" s="26" t="inlineStr"/>
       <c r="K41" s="26" t="inlineStr"/>
       <c r="L41" s="20" t="n"/>
       <c r="M41" s="20" t="n"/>
@@ -3457,24 +3508,24 @@
     <row r="42">
       <c r="A42" s="21" t="inlineStr">
         <is>
-          <t>5.2</t>
+          <t>6.7</t>
         </is>
       </c>
       <c r="B42" s="22" t="inlineStr">
         <is>
-          <t>Final revisions &amp; deliverable acceptance</t>
+          <t>Policy lifecycle, change process &amp; automation (policy-as-code, reviews)</t>
         </is>
       </c>
       <c r="C42" s="23" t="inlineStr">
         <is>
-          <t>Joint</t>
+          <t>Consultant</t>
         </is>
       </c>
       <c r="D42" s="24" t="n">
-        <v>46377</v>
+        <v>46328</v>
       </c>
       <c r="E42" s="24" t="n">
-        <v>46379</v>
+        <v>46360</v>
       </c>
       <c r="F42" s="21">
         <f>NETWORKDAYS(D42,E42,Inputs!$A$16:$A$21)</f>
@@ -3489,12 +3540,12 @@
       </c>
       <c r="I42" s="23" t="inlineStr">
         <is>
-          <t>5.1</t>
+          <t>5.3</t>
         </is>
       </c>
       <c r="J42" s="26" t="inlineStr">
         <is>
-          <t>Acceptance sign-off</t>
+          <t>Updated process docs</t>
         </is>
       </c>
       <c r="K42" s="26" t="inlineStr"/>
@@ -3516,49 +3567,45 @@
       <c r="AA42" s="20" t="n"/>
     </row>
     <row r="43">
-      <c r="A43" s="21" t="inlineStr">
-        <is>
-          <t>5.3</t>
-        </is>
-      </c>
-      <c r="B43" s="22" t="inlineStr">
-        <is>
-          <t>Knowledge transfer &amp; handover</t>
-        </is>
-      </c>
-      <c r="C43" s="23" t="inlineStr">
-        <is>
-          <t>Consultant</t>
-        </is>
-      </c>
-      <c r="D43" s="24" t="n">
-        <v>46384</v>
-      </c>
-      <c r="E43" s="24" t="n">
-        <v>46386</v>
-      </c>
-      <c r="F43" s="21">
+      <c r="A43" s="27" t="inlineStr">
+        <is>
+          <t>6.8</t>
+        </is>
+      </c>
+      <c r="B43" s="33" t="inlineStr">
+        <is>
+          <t>Milestone: Horizon 1 remediation complete</t>
+        </is>
+      </c>
+      <c r="C43" s="29" t="inlineStr">
+        <is>
+          <t>Joint</t>
+        </is>
+      </c>
+      <c r="D43" s="30" t="n">
+        <v>46374</v>
+      </c>
+      <c r="E43" s="30" t="n">
+        <v>46374</v>
+      </c>
+      <c r="F43" s="27">
         <f>NETWORKDAYS(D43,E43,Inputs!$A$16:$A$21)</f>
         <v/>
       </c>
-      <c r="G43" s="25" t="n">
+      <c r="G43" s="31" t="n">
         <v>0</v>
       </c>
-      <c r="H43" s="21">
+      <c r="H43" s="27">
         <f>IF(G43&gt;=1,"Complete",IF(E43&lt;Inputs!$B$7,"Late",IF(G43&gt;0,"In Progress",IF(D43&lt;=Inputs!$B$7,"Late Start","Not Started"))))</f>
         <v/>
       </c>
-      <c r="I43" s="23" t="inlineStr">
-        <is>
-          <t>5.2</t>
-        </is>
-      </c>
-      <c r="J43" s="26" t="inlineStr">
-        <is>
-          <t>Handover package</t>
-        </is>
-      </c>
-      <c r="K43" s="26" t="inlineStr"/>
+      <c r="I43" s="29" t="inlineStr">
+        <is>
+          <t>6.6</t>
+        </is>
+      </c>
+      <c r="J43" s="32" t="inlineStr"/>
+      <c r="K43" s="32" t="inlineStr"/>
       <c r="L43" s="20" t="n"/>
       <c r="M43" s="20" t="n"/>
       <c r="N43" s="20" t="n"/>
@@ -3577,49 +3624,40 @@
       <c r="AA43" s="20" t="n"/>
     </row>
     <row r="44">
-      <c r="A44" s="27" t="inlineStr">
-        <is>
-          <t>5.4</t>
-        </is>
-      </c>
-      <c r="B44" s="33" t="inlineStr">
-        <is>
-          <t>Milestone: Project close</t>
-        </is>
-      </c>
-      <c r="C44" s="29" t="inlineStr">
-        <is>
-          <t>Joint</t>
-        </is>
-      </c>
-      <c r="D44" s="30" t="n">
-        <v>46387</v>
-      </c>
-      <c r="E44" s="30" t="n">
-        <v>46387</v>
-      </c>
-      <c r="F44" s="27">
+      <c r="A44" s="17" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>Phase 7 – Validation &amp; Closeout</t>
+        </is>
+      </c>
+      <c r="C44" s="17" t="inlineStr"/>
+      <c r="D44" s="18">
+        <f>MIN(D45:D49)</f>
+        <v/>
+      </c>
+      <c r="E44" s="18">
+        <f>MAX(E45:E49)</f>
+        <v/>
+      </c>
+      <c r="F44" s="17">
         <f>NETWORKDAYS(D44,E44,Inputs!$A$16:$A$21)</f>
         <v/>
       </c>
-      <c r="G44" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="H44" s="27">
-        <f>IF(G44&gt;=1,"Complete",IF(E44&lt;Inputs!$B$7,"Late",IF(G44&gt;0,"In Progress",IF(D44&lt;=Inputs!$B$7,"Late Start","Not Started"))))</f>
-        <v/>
-      </c>
-      <c r="I44" s="29" t="inlineStr">
-        <is>
-          <t>5.3</t>
-        </is>
-      </c>
-      <c r="J44" s="32" t="inlineStr">
-        <is>
-          <t>Closeout report</t>
-        </is>
-      </c>
-      <c r="K44" s="32" t="inlineStr"/>
+      <c r="G44" s="19">
+        <f>IFERROR(SUMPRODUCT(F45:F49,G45:G49)/SUM(F45:F49),0)</f>
+        <v/>
+      </c>
+      <c r="H44" s="17">
+        <f>IF(G44&gt;=1,"Complete",IF(G44&gt;0,"In Progress","Not Started"))</f>
+        <v/>
+      </c>
+      <c r="I44" s="17" t="n"/>
+      <c r="J44" s="3" t="n"/>
+      <c r="K44" s="3" t="n"/>
       <c r="L44" s="20" t="n"/>
       <c r="M44" s="20" t="n"/>
       <c r="N44" s="20" t="n"/>
@@ -3637,91 +3675,392 @@
       <c r="Z44" s="20" t="n"/>
       <c r="AA44" s="20" t="n"/>
     </row>
+    <row r="45">
+      <c r="A45" s="21" t="inlineStr">
+        <is>
+          <t>7.1</t>
+        </is>
+      </c>
+      <c r="B45" s="22" t="inlineStr">
+        <is>
+          <t>Post-remediation validation, testing &amp; maturity re-score</t>
+        </is>
+      </c>
+      <c r="C45" s="23" t="inlineStr">
+        <is>
+          <t>Consultant</t>
+        </is>
+      </c>
+      <c r="D45" s="24" t="n">
+        <v>46370</v>
+      </c>
+      <c r="E45" s="24" t="n">
+        <v>46374</v>
+      </c>
+      <c r="F45" s="21">
+        <f>NETWORKDAYS(D45,E45,Inputs!$A$16:$A$21)</f>
+        <v/>
+      </c>
+      <c r="G45" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H45" s="21">
+        <f>IF(G45&gt;=1,"Complete",IF(E45&lt;Inputs!$B$7,"Late",IF(G45&gt;0,"In Progress",IF(D45&lt;=Inputs!$B$7,"Late Start","Not Started"))))</f>
+        <v/>
+      </c>
+      <c r="I45" s="23" t="inlineStr">
+        <is>
+          <t>6.5</t>
+        </is>
+      </c>
+      <c r="J45" s="26" t="inlineStr">
+        <is>
+          <t>Validation results</t>
+        </is>
+      </c>
+      <c r="K45" s="26" t="inlineStr"/>
+      <c r="L45" s="20" t="n"/>
+      <c r="M45" s="20" t="n"/>
+      <c r="N45" s="20" t="n"/>
+      <c r="O45" s="20" t="n"/>
+      <c r="P45" s="20" t="n"/>
+      <c r="Q45" s="20" t="n"/>
+      <c r="R45" s="20" t="n"/>
+      <c r="S45" s="20" t="n"/>
+      <c r="T45" s="20" t="n"/>
+      <c r="U45" s="20" t="n"/>
+      <c r="V45" s="20" t="n"/>
+      <c r="W45" s="20" t="n"/>
+      <c r="X45" s="20" t="n"/>
+      <c r="Y45" s="20" t="n"/>
+      <c r="Z45" s="20" t="n"/>
+      <c r="AA45" s="20" t="n"/>
+    </row>
     <row r="46">
-      <c r="A46" s="34" t="n"/>
-      <c r="B46" s="35" t="inlineStr">
+      <c r="A46" s="27" t="inlineStr">
+        <is>
+          <t>7.2</t>
+        </is>
+      </c>
+      <c r="B46" s="28" t="inlineStr">
+        <is>
+          <t>DELIVERABLE: Post-Remediation Report &amp; as-built architecture</t>
+        </is>
+      </c>
+      <c r="C46" s="29" t="inlineStr">
+        <is>
+          <t>Consultant</t>
+        </is>
+      </c>
+      <c r="D46" s="30" t="n">
+        <v>46372</v>
+      </c>
+      <c r="E46" s="30" t="n">
+        <v>46378</v>
+      </c>
+      <c r="F46" s="27">
+        <f>NETWORKDAYS(D46,E46,Inputs!$A$16:$A$21)</f>
+        <v/>
+      </c>
+      <c r="G46" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="H46" s="27">
+        <f>IF(G46&gt;=1,"Complete",IF(E46&lt;Inputs!$B$7,"Late",IF(G46&gt;0,"In Progress",IF(D46&lt;=Inputs!$B$7,"Late Start","Not Started"))))</f>
+        <v/>
+      </c>
+      <c r="I46" s="29" t="inlineStr">
+        <is>
+          <t>7.1</t>
+        </is>
+      </c>
+      <c r="J46" s="32" t="inlineStr">
+        <is>
+          <t>D5 – Post-Remediation Report</t>
+        </is>
+      </c>
+      <c r="K46" s="32" t="inlineStr"/>
+      <c r="L46" s="20" t="n"/>
+      <c r="M46" s="20" t="n"/>
+      <c r="N46" s="20" t="n"/>
+      <c r="O46" s="20" t="n"/>
+      <c r="P46" s="20" t="n"/>
+      <c r="Q46" s="20" t="n"/>
+      <c r="R46" s="20" t="n"/>
+      <c r="S46" s="20" t="n"/>
+      <c r="T46" s="20" t="n"/>
+      <c r="U46" s="20" t="n"/>
+      <c r="V46" s="20" t="n"/>
+      <c r="W46" s="20" t="n"/>
+      <c r="X46" s="20" t="n"/>
+      <c r="Y46" s="20" t="n"/>
+      <c r="Z46" s="20" t="n"/>
+      <c r="AA46" s="20" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="21" t="inlineStr">
+        <is>
+          <t>7.3</t>
+        </is>
+      </c>
+      <c r="B47" s="22" t="inlineStr">
+        <is>
+          <t>Knowledge transfer, runbooks &amp; handover</t>
+        </is>
+      </c>
+      <c r="C47" s="23" t="inlineStr">
+        <is>
+          <t>Consultant</t>
+        </is>
+      </c>
+      <c r="D47" s="24" t="n">
+        <v>46377</v>
+      </c>
+      <c r="E47" s="24" t="n">
+        <v>46379</v>
+      </c>
+      <c r="F47" s="21">
+        <f>NETWORKDAYS(D47,E47,Inputs!$A$16:$A$21)</f>
+        <v/>
+      </c>
+      <c r="G47" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H47" s="21">
+        <f>IF(G47&gt;=1,"Complete",IF(E47&lt;Inputs!$B$7,"Late",IF(G47&gt;0,"In Progress",IF(D47&lt;=Inputs!$B$7,"Late Start","Not Started"))))</f>
+        <v/>
+      </c>
+      <c r="I47" s="23" t="inlineStr">
+        <is>
+          <t>7.2</t>
+        </is>
+      </c>
+      <c r="J47" s="26" t="inlineStr">
+        <is>
+          <t>Handover package</t>
+        </is>
+      </c>
+      <c r="K47" s="26" t="inlineStr"/>
+      <c r="L47" s="20" t="n"/>
+      <c r="M47" s="20" t="n"/>
+      <c r="N47" s="20" t="n"/>
+      <c r="O47" s="20" t="n"/>
+      <c r="P47" s="20" t="n"/>
+      <c r="Q47" s="20" t="n"/>
+      <c r="R47" s="20" t="n"/>
+      <c r="S47" s="20" t="n"/>
+      <c r="T47" s="20" t="n"/>
+      <c r="U47" s="20" t="n"/>
+      <c r="V47" s="20" t="n"/>
+      <c r="W47" s="20" t="n"/>
+      <c r="X47" s="20" t="n"/>
+      <c r="Y47" s="20" t="n"/>
+      <c r="Z47" s="20" t="n"/>
+      <c r="AA47" s="20" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="21" t="inlineStr">
+        <is>
+          <t>7.4</t>
+        </is>
+      </c>
+      <c r="B48" s="22" t="inlineStr">
+        <is>
+          <t>Final status report &amp; closeout</t>
+        </is>
+      </c>
+      <c r="C48" s="23" t="inlineStr">
+        <is>
+          <t>Consultant</t>
+        </is>
+      </c>
+      <c r="D48" s="24" t="n">
+        <v>46384</v>
+      </c>
+      <c r="E48" s="24" t="n">
+        <v>46386</v>
+      </c>
+      <c r="F48" s="21">
+        <f>NETWORKDAYS(D48,E48,Inputs!$A$16:$A$21)</f>
+        <v/>
+      </c>
+      <c r="G48" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H48" s="21">
+        <f>IF(G48&gt;=1,"Complete",IF(E48&lt;Inputs!$B$7,"Late",IF(G48&gt;0,"In Progress",IF(D48&lt;=Inputs!$B$7,"Late Start","Not Started"))))</f>
+        <v/>
+      </c>
+      <c r="I48" s="23" t="inlineStr">
+        <is>
+          <t>7.3</t>
+        </is>
+      </c>
+      <c r="J48" s="26" t="inlineStr">
+        <is>
+          <t>Closeout report</t>
+        </is>
+      </c>
+      <c r="K48" s="26" t="inlineStr"/>
+      <c r="L48" s="20" t="n"/>
+      <c r="M48" s="20" t="n"/>
+      <c r="N48" s="20" t="n"/>
+      <c r="O48" s="20" t="n"/>
+      <c r="P48" s="20" t="n"/>
+      <c r="Q48" s="20" t="n"/>
+      <c r="R48" s="20" t="n"/>
+      <c r="S48" s="20" t="n"/>
+      <c r="T48" s="20" t="n"/>
+      <c r="U48" s="20" t="n"/>
+      <c r="V48" s="20" t="n"/>
+      <c r="W48" s="20" t="n"/>
+      <c r="X48" s="20" t="n"/>
+      <c r="Y48" s="20" t="n"/>
+      <c r="Z48" s="20" t="n"/>
+      <c r="AA48" s="20" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="27" t="inlineStr">
+        <is>
+          <t>7.5</t>
+        </is>
+      </c>
+      <c r="B49" s="33" t="inlineStr">
+        <is>
+          <t>Milestone: Project close</t>
+        </is>
+      </c>
+      <c r="C49" s="29" t="inlineStr">
+        <is>
+          <t>Joint</t>
+        </is>
+      </c>
+      <c r="D49" s="30" t="n">
+        <v>46387</v>
+      </c>
+      <c r="E49" s="30" t="n">
+        <v>46387</v>
+      </c>
+      <c r="F49" s="27">
+        <f>NETWORKDAYS(D49,E49,Inputs!$A$16:$A$21)</f>
+        <v/>
+      </c>
+      <c r="G49" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="H49" s="27">
+        <f>IF(G49&gt;=1,"Complete",IF(E49&lt;Inputs!$B$7,"Late",IF(G49&gt;0,"In Progress",IF(D49&lt;=Inputs!$B$7,"Late Start","Not Started"))))</f>
+        <v/>
+      </c>
+      <c r="I49" s="29" t="inlineStr">
+        <is>
+          <t>7.4</t>
+        </is>
+      </c>
+      <c r="J49" s="32" t="inlineStr"/>
+      <c r="K49" s="32" t="inlineStr"/>
+      <c r="L49" s="20" t="n"/>
+      <c r="M49" s="20" t="n"/>
+      <c r="N49" s="20" t="n"/>
+      <c r="O49" s="20" t="n"/>
+      <c r="P49" s="20" t="n"/>
+      <c r="Q49" s="20" t="n"/>
+      <c r="R49" s="20" t="n"/>
+      <c r="S49" s="20" t="n"/>
+      <c r="T49" s="20" t="n"/>
+      <c r="U49" s="20" t="n"/>
+      <c r="V49" s="20" t="n"/>
+      <c r="W49" s="20" t="n"/>
+      <c r="X49" s="20" t="n"/>
+      <c r="Y49" s="20" t="n"/>
+      <c r="Z49" s="20" t="n"/>
+      <c r="AA49" s="20" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="34" t="n"/>
+      <c r="B51" s="35" t="inlineStr">
         <is>
           <t>OVERALL ENGAGEMENT</t>
         </is>
       </c>
-      <c r="C46" s="34" t="n"/>
-      <c r="D46" s="36">
-        <f>MIN(D5:D44)</f>
-        <v/>
-      </c>
-      <c r="E46" s="36">
-        <f>MAX(E5:E44)</f>
-        <v/>
-      </c>
-      <c r="F46" s="34">
-        <f>NETWORKDAYS(D46,E46,Inputs!$A$16:$A$21)</f>
-        <v/>
-      </c>
-      <c r="G46" s="37">
-        <f>IFERROR((F5*G5+F10*G10+F19*G19+F27*G27+F34*G34+F40*G40)/(F5+F10+F19+F27+F34+F40),0)</f>
-        <v/>
-      </c>
-      <c r="H46" s="34" t="n"/>
-      <c r="I46" s="34" t="n"/>
-      <c r="J46" s="34" t="n"/>
-      <c r="K46" s="34" t="n"/>
-    </row>
-    <row r="48">
-      <c r="B48" s="15" t="inlineStr">
+      <c r="C51" s="34" t="n"/>
+      <c r="D51" s="36">
+        <f>MIN(D5:D49)</f>
+        <v/>
+      </c>
+      <c r="E51" s="36">
+        <f>MAX(E5:E49)</f>
+        <v/>
+      </c>
+      <c r="F51" s="34">
+        <f>NETWORKDAYS(D51,E51,Inputs!$A$16:$A$21)</f>
+        <v/>
+      </c>
+      <c r="G51" s="37">
+        <f>IFERROR((F5*G5+F10*G10+F17*G17+F23*G23+F27*G27+F31*G31+F35*G35+F44*G44)/(F5+F10+F17+F23+F27+F31+F35+F44),0)</f>
+        <v/>
+      </c>
+      <c r="H51" s="34" t="n"/>
+      <c r="I51" s="34" t="n"/>
+      <c r="J51" s="34" t="n"/>
+      <c r="K51" s="34" t="n"/>
+    </row>
+    <row r="53">
+      <c r="B53" s="15" t="inlineStr">
         <is>
           <t>Gantt legend:</t>
         </is>
       </c>
     </row>
-    <row r="49">
-      <c r="B49" s="38" t="inlineStr">
+    <row r="54">
+      <c r="B54" s="38" t="inlineStr">
         <is>
           <t>Phase</t>
         </is>
       </c>
-      <c r="C49" s="39" t="n"/>
-    </row>
-    <row r="50">
-      <c r="B50" s="38" t="inlineStr">
+      <c r="C54" s="39" t="n"/>
+    </row>
+    <row r="55">
+      <c r="B55" s="38" t="inlineStr">
         <is>
           <t>Task</t>
         </is>
       </c>
-      <c r="C50" s="40" t="n"/>
-    </row>
-    <row r="51">
-      <c r="B51" s="38" t="inlineStr">
+      <c r="C55" s="40" t="n"/>
+    </row>
+    <row r="56">
+      <c r="B56" s="38" t="inlineStr">
         <is>
           <t>Deliverable</t>
         </is>
       </c>
-      <c r="C51" s="41" t="n"/>
-    </row>
-    <row r="52">
-      <c r="B52" s="38" t="inlineStr">
+      <c r="C56" s="41" t="n"/>
+    </row>
+    <row r="57">
+      <c r="B57" s="38" t="inlineStr">
         <is>
           <t>Milestone</t>
         </is>
       </c>
-      <c r="C52" s="42" t="n"/>
-    </row>
-    <row r="53">
-      <c r="B53" s="38" t="inlineStr">
+      <c r="C57" s="42" t="n"/>
+    </row>
+    <row r="58">
+      <c r="B58" s="38" t="inlineStr">
         <is>
           <t>Current week (header)</t>
         </is>
       </c>
-      <c r="C53" s="43" t="n"/>
-    </row>
-    <row r="55">
-      <c r="B55" s="13" t="inlineStr">
+      <c r="C58" s="43" t="n"/>
+    </row>
+    <row r="60">
+      <c r="B60" s="13" t="inlineStr">
         <is>
           <t>% Complete values reflect status as of Sep 28, 2026 (week 3) – update weekly.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="L5:AA44">
+  <conditionalFormatting sqref="L5:AA49">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>AND($D5&lt;=L$4+4,$E5&gt;=L$4,LEFT($B5,9)="Milestone")</formula>
     </cfRule>
@@ -3740,7 +4079,7 @@
       <formula>AND(Inputs!$B$7&gt;=L$4,Inputs!$B$7&lt;=L$4+6)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H5:H44">
+  <conditionalFormatting sqref="H5:H49">
     <cfRule type="expression" priority="6" dxfId="5">
       <formula>$H5="Complete"</formula>
     </cfRule>
@@ -3754,7 +4093,7 @@
       <formula>$H5="Late Start"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G5:G44">
+  <conditionalFormatting sqref="G5:G49">
     <cfRule type="dataBar" priority="10">
       <dataBar>
         <cfvo type="num" val="0"/>
@@ -3764,11 +4103,11 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="G5:G44" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" error="Enter 0%–100%" type="decimal" operator="between">
+    <dataValidation sqref="G5:G49" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" error="Enter 0%–100%" type="decimal" operator="between">
       <formula1>0</formula1>
       <formula2>1</formula2>
     </dataValidation>
-    <dataValidation sqref="C5:C44" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="C5:C49" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Consultant,Client,Joint"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3783,7 +4122,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -3874,15 +4213,15 @@
       </c>
       <c r="E4" s="21" t="inlineStr">
         <is>
-          <t>1.7</t>
+          <t>1.6</t>
         </is>
       </c>
       <c r="F4" s="46">
-        <f>WORKDAY('Project Plan'!E17,-3,Inputs!$A$16:$A$21)</f>
+        <f>WORKDAY('Project Plan'!E16,-1,Inputs!$A$16:$A$21)</f>
         <v/>
       </c>
       <c r="G4" s="47">
-        <f>'Project Plan'!E17</f>
+        <f>'Project Plan'!E16</f>
         <v/>
       </c>
       <c r="H4" s="48" t="inlineStr">
@@ -3891,7 +4230,7 @@
         </is>
       </c>
       <c r="I4" s="11">
-        <f>'Project Plan'!H17</f>
+        <f>'Project Plan'!H16</f>
         <v/>
       </c>
     </row>
@@ -3918,15 +4257,15 @@
       </c>
       <c r="E5" s="21" t="inlineStr">
         <is>
-          <t>2.6</t>
+          <t>2.5</t>
         </is>
       </c>
       <c r="F5" s="46">
-        <f>WORKDAY('Project Plan'!E25,-3,Inputs!$A$16:$A$21)</f>
+        <f>WORKDAY('Project Plan'!E22,-1,Inputs!$A$16:$A$21)</f>
         <v/>
       </c>
       <c r="G5" s="47">
-        <f>'Project Plan'!E25</f>
+        <f>'Project Plan'!E22</f>
         <v/>
       </c>
       <c r="H5" s="48" t="inlineStr">
@@ -3935,7 +4274,7 @@
         </is>
       </c>
       <c r="I5" s="11">
-        <f>'Project Plan'!H25</f>
+        <f>'Project Plan'!H22</f>
         <v/>
       </c>
     </row>
@@ -3952,7 +4291,7 @@
       </c>
       <c r="C6" s="45" t="inlineStr">
         <is>
-          <t>Future-state vision &amp; target architecture; remediation initiatives mapped to gaps; prioritization; phased sequencing (0–6/6–12/12–24 mo); budget ranges, resourcing, KPIs.</t>
+          <t>Future-state vision &amp; target architecture; remediation initiatives mapped to gaps; prioritization; phased sequencing (0–3 / 3–12 / 12–24 mo); budget ranges, resourcing, KPIs.</t>
         </is>
       </c>
       <c r="D6" s="26" t="inlineStr">
@@ -3962,15 +4301,15 @@
       </c>
       <c r="E6" s="21" t="inlineStr">
         <is>
-          <t>4.5</t>
+          <t>4.2</t>
         </is>
       </c>
       <c r="F6" s="46">
-        <f>WORKDAY('Project Plan'!E39,-3,Inputs!$A$16:$A$21)</f>
+        <f>WORKDAY('Project Plan'!E29,-1,Inputs!$A$16:$A$21)</f>
         <v/>
       </c>
       <c r="G6" s="47">
-        <f>'Project Plan'!E39</f>
+        <f>'Project Plan'!E29</f>
         <v/>
       </c>
       <c r="H6" s="48" t="inlineStr">
@@ -3979,7 +4318,7 @@
         </is>
       </c>
       <c r="I6" s="11">
-        <f>'Project Plan'!H39</f>
+        <f>'Project Plan'!H29</f>
         <v/>
       </c>
     </row>
@@ -3996,7 +4335,7 @@
       </c>
       <c r="C7" s="45" t="inlineStr">
         <is>
-          <t>Summary of findings, future state and roadmap for steering committee.</t>
+          <t>Presentation of D1, D2 and D3 to steering committee; approval to proceed with remediation.</t>
         </is>
       </c>
       <c r="D7" s="26" t="inlineStr">
@@ -4006,31 +4345,119 @@
       </c>
       <c r="E7" s="21" t="inlineStr">
         <is>
+          <t>4.3</t>
+        </is>
+      </c>
+      <c r="F7" s="46">
+        <f>WORKDAY('Project Plan'!E30,-1,Inputs!$A$16:$A$21)</f>
+        <v/>
+      </c>
+      <c r="G7" s="47">
+        <f>'Project Plan'!E30</f>
+        <v/>
+      </c>
+      <c r="H7" s="48" t="inlineStr">
+        <is>
+          <t>Executive Sponsor</t>
+        </is>
+      </c>
+      <c r="I7" s="11">
+        <f>'Project Plan'!H30</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8" ht="62" customHeight="1">
+      <c r="A8" s="21" t="inlineStr">
+        <is>
+          <t>D4</t>
+        </is>
+      </c>
+      <c r="B8" s="44" t="inlineStr">
+        <is>
+          <t>Remediation Execution Plan</t>
+        </is>
+      </c>
+      <c r="C8" s="45" t="inlineStr">
+        <is>
+          <t>Detailed work packages, change windows, CAB schedule, rollback and test plans for in-engagement remediation.</t>
+        </is>
+      </c>
+      <c r="D8" s="26" t="inlineStr">
+        <is>
+          <t>Excel + Word</t>
+        </is>
+      </c>
+      <c r="E8" s="21" t="inlineStr">
+        <is>
           <t>5.1</t>
         </is>
       </c>
-      <c r="F7" s="46">
-        <f>WORKDAY('Project Plan'!E41,-3,Inputs!$A$16:$A$21)</f>
-        <v/>
-      </c>
-      <c r="G7" s="47">
-        <f>'Project Plan'!E41</f>
-        <v/>
-      </c>
-      <c r="H7" s="48" t="inlineStr">
-        <is>
-          <t>Executive Sponsor</t>
-        </is>
-      </c>
-      <c r="I7" s="11">
-        <f>'Project Plan'!H41</f>
-        <v/>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="13" t="inlineStr">
-        <is>
-          <t>Draft Due = 3 working days before final (assumption: client review window). Green = linked to Project Plan.</t>
+      <c r="F8" s="46">
+        <f>WORKDAY('Project Plan'!E32,-1,Inputs!$A$16:$A$21)</f>
+        <v/>
+      </c>
+      <c r="G8" s="47">
+        <f>'Project Plan'!E32</f>
+        <v/>
+      </c>
+      <c r="H8" s="48" t="inlineStr">
+        <is>
+          <t>Network Security Lead</t>
+        </is>
+      </c>
+      <c r="I8" s="11">
+        <f>'Project Plan'!H32</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9" ht="62" customHeight="1">
+      <c r="A9" s="21" t="inlineStr">
+        <is>
+          <t>D5</t>
+        </is>
+      </c>
+      <c r="B9" s="44" t="inlineStr">
+        <is>
+          <t>Post-Remediation Report</t>
+        </is>
+      </c>
+      <c r="C9" s="45" t="inlineStr">
+        <is>
+          <t>Validation results, maturity re-score vs. baseline, as-built architecture, remaining roadmap items.</t>
+        </is>
+      </c>
+      <c r="D9" s="26" t="inlineStr">
+        <is>
+          <t>Word/PDF + Visio</t>
+        </is>
+      </c>
+      <c r="E9" s="21" t="inlineStr">
+        <is>
+          <t>7.2</t>
+        </is>
+      </c>
+      <c r="F9" s="46">
+        <f>WORKDAY('Project Plan'!E46,-1,Inputs!$A$16:$A$21)</f>
+        <v/>
+      </c>
+      <c r="G9" s="47">
+        <f>'Project Plan'!E46</f>
+        <v/>
+      </c>
+      <c r="H9" s="48" t="inlineStr">
+        <is>
+          <t>CISO</t>
+        </is>
+      </c>
+      <c r="I9" s="11">
+        <f>'Project Plan'!H46</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="13" t="inlineStr">
+        <is>
+          <t>Draft Due = 1 working day before final (assumption: client review window). Green = linked to Project Plan.</t>
         </is>
       </c>
     </row>
@@ -4045,7 +4472,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -4115,15 +4542,15 @@
     <row r="5">
       <c r="A5" s="21" t="inlineStr">
         <is>
-          <t>1.8</t>
+          <t>1.6</t>
         </is>
       </c>
       <c r="B5" s="9">
-        <f>'Project Plan'!B18</f>
+        <f>'Project Plan'!B16</f>
         <v/>
       </c>
       <c r="C5" s="49">
-        <f>'Project Plan'!E18</f>
+        <f>'Project Plan'!E16</f>
         <v/>
       </c>
       <c r="D5" s="50">
@@ -4131,22 +4558,22 @@
         <v/>
       </c>
       <c r="E5" s="11">
-        <f>'Project Plan'!H18</f>
+        <f>'Project Plan'!H16</f>
         <v/>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="21" t="inlineStr">
         <is>
-          <t>2.7</t>
+          <t>2.5</t>
         </is>
       </c>
       <c r="B6" s="9">
-        <f>'Project Plan'!B26</f>
+        <f>'Project Plan'!B22</f>
         <v/>
       </c>
       <c r="C6" s="49">
-        <f>'Project Plan'!E26</f>
+        <f>'Project Plan'!E22</f>
         <v/>
       </c>
       <c r="D6" s="50">
@@ -4154,22 +4581,22 @@
         <v/>
       </c>
       <c r="E6" s="11">
-        <f>'Project Plan'!H26</f>
+        <f>'Project Plan'!H22</f>
         <v/>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="21" t="inlineStr">
         <is>
-          <t>3.6</t>
+          <t>4.2</t>
         </is>
       </c>
       <c r="B7" s="9">
-        <f>'Project Plan'!B33</f>
+        <f>'Project Plan'!B29</f>
         <v/>
       </c>
       <c r="C7" s="49">
-        <f>'Project Plan'!E33</f>
+        <f>'Project Plan'!E29</f>
         <v/>
       </c>
       <c r="D7" s="50">
@@ -4177,22 +4604,22 @@
         <v/>
       </c>
       <c r="E7" s="11">
-        <f>'Project Plan'!H33</f>
+        <f>'Project Plan'!H29</f>
         <v/>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="21" t="inlineStr">
         <is>
-          <t>4.5</t>
+          <t>4.3</t>
         </is>
       </c>
       <c r="B8" s="9">
-        <f>'Project Plan'!B39</f>
+        <f>'Project Plan'!B30</f>
         <v/>
       </c>
       <c r="C8" s="49">
-        <f>'Project Plan'!E39</f>
+        <f>'Project Plan'!E30</f>
         <v/>
       </c>
       <c r="D8" s="50">
@@ -4200,22 +4627,22 @@
         <v/>
       </c>
       <c r="E8" s="11">
-        <f>'Project Plan'!H39</f>
+        <f>'Project Plan'!H30</f>
         <v/>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="21" t="inlineStr">
         <is>
-          <t>5.1</t>
+          <t>5.3</t>
         </is>
       </c>
       <c r="B9" s="9">
-        <f>'Project Plan'!B41</f>
+        <f>'Project Plan'!B34</f>
         <v/>
       </c>
       <c r="C9" s="49">
-        <f>'Project Plan'!E41</f>
+        <f>'Project Plan'!E34</f>
         <v/>
       </c>
       <c r="D9" s="50">
@@ -4223,22 +4650,22 @@
         <v/>
       </c>
       <c r="E9" s="11">
-        <f>'Project Plan'!H41</f>
+        <f>'Project Plan'!H34</f>
         <v/>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="21" t="inlineStr">
         <is>
-          <t>5.4</t>
+          <t>6.8</t>
         </is>
       </c>
       <c r="B10" s="9">
-        <f>'Project Plan'!B44</f>
+        <f>'Project Plan'!B43</f>
         <v/>
       </c>
       <c r="C10" s="49">
-        <f>'Project Plan'!E44</f>
+        <f>'Project Plan'!E43</f>
         <v/>
       </c>
       <c r="D10" s="50">
@@ -4246,7 +4673,53 @@
         <v/>
       </c>
       <c r="E10" s="11">
-        <f>'Project Plan'!H44</f>
+        <f>'Project Plan'!H43</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="21" t="inlineStr">
+        <is>
+          <t>7.2</t>
+        </is>
+      </c>
+      <c r="B11" s="9">
+        <f>'Project Plan'!B46</f>
+        <v/>
+      </c>
+      <c r="C11" s="49">
+        <f>'Project Plan'!E46</f>
+        <v/>
+      </c>
+      <c r="D11" s="50">
+        <f>C11-Inputs!$B$7</f>
+        <v/>
+      </c>
+      <c r="E11" s="11">
+        <f>'Project Plan'!H46</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="21" t="inlineStr">
+        <is>
+          <t>7.5</t>
+        </is>
+      </c>
+      <c r="B12" s="9">
+        <f>'Project Plan'!B49</f>
+        <v/>
+      </c>
+      <c r="C12" s="49">
+        <f>'Project Plan'!E49</f>
+        <v/>
+      </c>
+      <c r="D12" s="50">
+        <f>C12-Inputs!$B$7</f>
+        <v/>
+      </c>
+      <c r="E12" s="11">
+        <f>'Project Plan'!H49</f>
         <v/>
       </c>
     </row>
@@ -4261,7 +4734,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G14"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -4431,7 +4904,7 @@
     <row r="7">
       <c r="A7" s="51" t="inlineStr">
         <is>
-          <t>Gap analysis &amp; maturity scoring</t>
+          <t>D2 Problem Areas &amp; Gaps Assessment</t>
         </is>
       </c>
       <c r="B7" s="52" t="inlineStr">
@@ -4449,9 +4922,9 @@
           <t>R</t>
         </is>
       </c>
-      <c r="E7" s="54" t="inlineStr">
-        <is>
-          <t>I</t>
+      <c r="E7" s="53" t="inlineStr">
+        <is>
+          <t>C</t>
         </is>
       </c>
       <c r="F7" s="53" t="inlineStr">
@@ -4468,27 +4941,27 @@
     <row r="8">
       <c r="A8" s="51" t="inlineStr">
         <is>
-          <t>D2 Problem Areas &amp; Gaps Assessment</t>
-        </is>
-      </c>
-      <c r="B8" s="52" t="inlineStr">
+          <t>Future-state vision</t>
+        </is>
+      </c>
+      <c r="B8" s="55" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="C8" s="55" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="D8" s="53" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="E8" s="52" t="inlineStr">
         <is>
           <t>A</t>
-        </is>
-      </c>
-      <c r="C8" s="55" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="D8" s="55" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="E8" s="53" t="inlineStr">
-        <is>
-          <t>C</t>
         </is>
       </c>
       <c r="F8" s="53" t="inlineStr">
@@ -4505,27 +4978,27 @@
     <row r="9">
       <c r="A9" s="51" t="inlineStr">
         <is>
-          <t>Future-state vision</t>
-        </is>
-      </c>
-      <c r="B9" s="55" t="inlineStr">
+          <t>D3 Modernization Roadmap</t>
+        </is>
+      </c>
+      <c r="B9" s="52" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C9" s="55" t="inlineStr">
         <is>
           <t>R</t>
         </is>
       </c>
-      <c r="C9" s="55" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
       <c r="D9" s="53" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="E9" s="52" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="E9" s="53" t="inlineStr">
+        <is>
+          <t>C</t>
         </is>
       </c>
       <c r="F9" s="53" t="inlineStr">
@@ -4533,16 +5006,16 @@
           <t>C</t>
         </is>
       </c>
-      <c r="G9" s="53" t="inlineStr">
-        <is>
-          <t>C</t>
+      <c r="G9" s="54" t="inlineStr">
+        <is>
+          <t>I</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="51" t="inlineStr">
         <is>
-          <t>Remediation plan &amp; prioritization</t>
+          <t>Executive readout (D1–D3)</t>
         </is>
       </c>
       <c r="B10" s="55" t="inlineStr">
@@ -4550,36 +5023,36 @@
           <t>R</t>
         </is>
       </c>
-      <c r="C10" s="55" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="D10" s="53" t="inlineStr">
+      <c r="C10" s="53" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
+      <c r="D10" s="54" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
       <c r="E10" s="52" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="F10" s="53" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="G10" s="53" t="inlineStr">
-        <is>
-          <t>C</t>
+      <c r="F10" s="54" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G10" s="54" t="inlineStr">
+        <is>
+          <t>I</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="51" t="inlineStr">
         <is>
-          <t>D3 Modernization Roadmap</t>
+          <t>D4 Remediation Execution Plan</t>
         </is>
       </c>
       <c r="B11" s="52" t="inlineStr">
@@ -4602,56 +5075,93 @@
           <t>C</t>
         </is>
       </c>
-      <c r="F11" s="53" t="inlineStr">
+      <c r="F11" s="55" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="G11" s="53" t="inlineStr">
         <is>
           <t>C</t>
-        </is>
-      </c>
-      <c r="G11" s="54" t="inlineStr">
-        <is>
-          <t>I</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="51" t="inlineStr">
         <is>
-          <t>Executive readout &amp; acceptance</t>
-        </is>
-      </c>
-      <c r="B12" s="55" t="inlineStr">
+          <t>Remediation execution &amp; change implementation</t>
+        </is>
+      </c>
+      <c r="B12" s="52" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C12" s="55" t="inlineStr">
         <is>
           <t>R</t>
         </is>
       </c>
-      <c r="C12" s="53" t="inlineStr">
+      <c r="D12" s="55" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="E12" s="54" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="F12" s="55" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="G12" s="53" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="D12" s="54" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="E12" s="52" t="inlineStr">
+    </row>
+    <row r="13">
+      <c r="A13" s="51" t="inlineStr">
+        <is>
+          <t>Validation &amp; D5 Post-Remediation Report</t>
+        </is>
+      </c>
+      <c r="B13" s="52" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="F12" s="54" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="G12" s="54" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="13" t="inlineStr">
+      <c r="C13" s="55" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="D13" s="55" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="E13" s="53" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="F13" s="53" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="G13" s="53" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="13" t="inlineStr">
         <is>
           <t>R = Responsible · A = Accountable · C = Consulted · I = Informed</t>
         </is>
@@ -4668,7 +5178,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J9"/>
+  <dimension ref="A1:J10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -4847,14 +5357,14 @@
       </c>
       <c r="C6" s="26" t="inlineStr">
         <is>
-          <t>Holiday period (Thanksgiving, late Dec) compresses review cycles</t>
+          <t>Compressed 4-week assessment limits review time for D1–D3</t>
         </is>
       </c>
       <c r="D6" s="23" t="n">
+        <v>4</v>
+      </c>
+      <c r="E6" s="23" t="n">
         <v>3</v>
-      </c>
-      <c r="E6" s="23" t="n">
-        <v>4</v>
       </c>
       <c r="F6" s="21">
         <f>D6*E6</f>
@@ -4866,7 +5376,7 @@
       </c>
       <c r="H6" s="26" t="inlineStr">
         <is>
-          <t>Front-load drafts; lock readout date by Nov 1</t>
+          <t>Daily working sessions; pre-schedule readout for Oct 9; drafts shared incrementally</t>
         </is>
       </c>
       <c r="I6" s="48" t="inlineStr">
@@ -4893,11 +5403,11 @@
       </c>
       <c r="C7" s="26" t="inlineStr">
         <is>
-          <t>Scope creep into implementation/remediation execution</t>
+          <t>Remediation changes cause outages or business disruption</t>
         </is>
       </c>
       <c r="D7" s="23" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E7" s="23" t="n">
         <v>2</v>
@@ -4912,12 +5422,12 @@
       </c>
       <c r="H7" s="26" t="inlineStr">
         <is>
-          <t>Change control per SOW; log out-of-scope asks</t>
+          <t>CAB approval, maintenance windows, tested rollback, staged rollout</t>
         </is>
       </c>
       <c r="I7" s="48" t="inlineStr">
         <is>
-          <t>Engagement Lead</t>
+          <t>NGFW Architect</t>
         </is>
       </c>
       <c r="J7" s="23" t="inlineStr">
@@ -4929,7 +5439,7 @@
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="21" t="inlineStr">
         <is>
-          <t>R5</t>
+          <t>R6</t>
         </is>
       </c>
       <c r="B8" s="23" t="inlineStr">
@@ -4939,14 +5449,14 @@
       </c>
       <c r="C8" s="26" t="inlineStr">
         <is>
-          <t>Incomplete CMDB / undocumented firewalls (shadow estate)</t>
+          <t>Limited change windows / holiday change freeze (late Nov, Dec)</t>
         </is>
       </c>
       <c r="D8" s="23" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E8" s="23" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F8" s="21">
         <f>D8*E8</f>
@@ -4958,12 +5468,12 @@
       </c>
       <c r="H8" s="26" t="inlineStr">
         <is>
-          <t>Validate inventory against network scans &amp; routing tables</t>
+          <t>Front-load high-impact changes Oct–mid Nov; confirm freeze dates</t>
         </is>
       </c>
       <c r="I8" s="48" t="inlineStr">
         <is>
-          <t>NGFW Architect</t>
+          <t>Client</t>
         </is>
       </c>
       <c r="J8" s="23" t="inlineStr">
@@ -4975,24 +5485,24 @@
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="21" t="inlineStr">
         <is>
-          <t>I1</t>
+          <t>R5</t>
         </is>
       </c>
       <c r="B9" s="23" t="inlineStr">
         <is>
-          <t>Issue</t>
+          <t>Risk</t>
         </is>
       </c>
       <c r="C9" s="26" t="inlineStr">
         <is>
-          <t>Config export for cloud firewalls pending security approval</t>
+          <t>Incomplete CMDB / undocumented firewalls (shadow estate)</t>
         </is>
       </c>
       <c r="D9" s="23" t="n">
         <v>3</v>
       </c>
       <c r="E9" s="23" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F9" s="21">
         <f>D9*E9</f>
@@ -5004,15 +5514,61 @@
       </c>
       <c r="H9" s="26" t="inlineStr">
         <is>
+          <t>Validate inventory against network scans &amp; routing tables</t>
+        </is>
+      </c>
+      <c r="I9" s="48" t="inlineStr">
+        <is>
+          <t>NGFW Architect</t>
+        </is>
+      </c>
+      <c r="J9" s="23" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="21" t="inlineStr">
+        <is>
+          <t>I1</t>
+        </is>
+      </c>
+      <c r="B10" s="23" t="inlineStr">
+        <is>
+          <t>Issue</t>
+        </is>
+      </c>
+      <c r="C10" s="26" t="inlineStr">
+        <is>
+          <t>Config export for cloud firewalls pending security approval</t>
+        </is>
+      </c>
+      <c r="D10" s="23" t="n">
+        <v>3</v>
+      </c>
+      <c r="E10" s="23" t="n">
+        <v>5</v>
+      </c>
+      <c r="F10" s="21">
+        <f>D10*E10</f>
+        <v/>
+      </c>
+      <c r="G10" s="21">
+        <f>IF(F10&gt;=15,"High",IF(F10&gt;=8,"Medium","Low"))</f>
+        <v/>
+      </c>
+      <c r="H10" s="26" t="inlineStr">
+        <is>
           <t>Sponsor escalation requested</t>
         </is>
       </c>
-      <c r="I9" s="48" t="inlineStr">
+      <c r="I10" s="48" t="inlineStr">
         <is>
           <t>Client</t>
         </is>
       </c>
-      <c r="J9" s="23" t="inlineStr">
+      <c r="J10" s="23" t="inlineStr">
         <is>
           <t>Open</t>
         </is>

</xml_diff>